<commit_message>
Update Customer_Requirement_Report.xlsx — Summary Timeline now a Gantt chart
Fresh web export: Summary timeline rendered as Month/Week Gantt grid
with colored markers (HumanSoft blue / Client orange / Go-live).
</commit_message>
<xml_diff>
--- a/Customer_Requirement_Report.xlsx
+++ b/Customer_Requirement_Report.xlsx
@@ -265,7 +265,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="12">
     <border>
       <left/>
       <right/>
@@ -287,11 +287,119 @@
         <color rgb="00E5E7EB"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00E5E7EB"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00E5E7EB"/>
+      </right>
+      <top style="thin">
+        <color rgb="00E5E7EB"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00E5E7EB"/>
+      </right>
+      <top style="thin">
+        <color rgb="00E5E7EB"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00E5E7EB"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00E5E7EB"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00E5E7EB"/>
+      </left>
+      <right style="thin">
+        <color rgb="00E5E7EB"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00E5E7EB"/>
+      </left>
+      <right style="thin">
+        <color rgb="00E5E7EB"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00E5E7EB"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00E5E7EB"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00E5E7EB"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00E5E7EB"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00E5E7EB"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00E5E7EB"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00E5E7EB"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00E5E7EB"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="61">
+  <cellXfs count="68">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -451,6 +559,13 @@
     <xf numFmtId="0" fontId="12" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -843,11 +958,6 @@
           <t>HumanSoft</t>
         </is>
       </c>
-      <c r="G2" s="3" t="n"/>
-      <c r="H2" s="3" t="n"/>
-      <c r="I2" s="3" t="n"/>
-      <c r="J2" s="3" t="n"/>
-      <c r="K2" s="3" t="n"/>
     </row>
     <row r="3">
       <c r="F3" s="4" t="inlineStr">
@@ -855,11 +965,6 @@
           <t>FM-SE-03</t>
         </is>
       </c>
-      <c r="G3" s="3" t="n"/>
-      <c r="H3" s="3" t="n"/>
-      <c r="I3" s="3" t="n"/>
-      <c r="J3" s="3" t="n"/>
-      <c r="K3" s="3" t="n"/>
     </row>
     <row r="4">
       <c r="F4" s="5" t="inlineStr">
@@ -867,11 +972,6 @@
           <t>วันที่เริ่มใช้/ แก้ไข : 02 กุมภาพันธ์ 2569/ 00</t>
         </is>
       </c>
-      <c r="G4" s="3" t="n"/>
-      <c r="H4" s="3" t="n"/>
-      <c r="I4" s="3" t="n"/>
-      <c r="J4" s="3" t="n"/>
-      <c r="K4" s="3" t="n"/>
     </row>
     <row r="6" ht="18" customHeight="1">
       <c r="A6" s="6" t="inlineStr">
@@ -879,20 +979,11 @@
           <t>Domain</t>
         </is>
       </c>
-      <c r="B6" s="7" t="n"/>
       <c r="C6" s="8" t="inlineStr">
         <is>
           <t>ทดสอบ</t>
         </is>
       </c>
-      <c r="D6" s="7" t="n"/>
-      <c r="E6" s="7" t="n"/>
-      <c r="F6" s="7" t="n"/>
-      <c r="G6" s="7" t="n"/>
-      <c r="H6" s="7" t="n"/>
-      <c r="I6" s="7" t="n"/>
-      <c r="J6" s="7" t="n"/>
-      <c r="K6" s="7" t="n"/>
     </row>
     <row r="7" ht="18" customHeight="1">
       <c r="A7" s="6" t="inlineStr">
@@ -900,20 +991,11 @@
           <t>บริษัท (Company)</t>
         </is>
       </c>
-      <c r="B7" s="7" t="n"/>
       <c r="C7" s="8" t="inlineStr">
         <is>
           <t>ทดสอบ</t>
         </is>
       </c>
-      <c r="D7" s="7" t="n"/>
-      <c r="E7" s="7" t="n"/>
-      <c r="F7" s="7" t="n"/>
-      <c r="G7" s="7" t="n"/>
-      <c r="H7" s="7" t="n"/>
-      <c r="I7" s="7" t="n"/>
-      <c r="J7" s="7" t="n"/>
-      <c r="K7" s="7" t="n"/>
     </row>
     <row r="8" ht="18" customHeight="1">
       <c r="A8" s="6" t="inlineStr">
@@ -921,20 +1003,11 @@
           <t>วันที่อัปเดต</t>
         </is>
       </c>
-      <c r="B8" s="7" t="n"/>
       <c r="C8" s="8" t="inlineStr">
         <is>
           <t>23/5/2026</t>
         </is>
       </c>
-      <c r="D8" s="7" t="n"/>
-      <c r="E8" s="7" t="n"/>
-      <c r="F8" s="7" t="n"/>
-      <c r="G8" s="7" t="n"/>
-      <c r="H8" s="7" t="n"/>
-      <c r="I8" s="7" t="n"/>
-      <c r="J8" s="7" t="n"/>
-      <c r="K8" s="7" t="n"/>
     </row>
     <row r="10" ht="22" customHeight="1">
       <c r="A10" s="9" t="inlineStr">
@@ -942,16 +1015,6 @@
           <t xml:space="preserve">    🎯  สรุป Pain Point หลัก</t>
         </is>
       </c>
-      <c r="B10" s="10" t="n"/>
-      <c r="C10" s="10" t="n"/>
-      <c r="D10" s="10" t="n"/>
-      <c r="E10" s="10" t="n"/>
-      <c r="F10" s="10" t="n"/>
-      <c r="G10" s="10" t="n"/>
-      <c r="H10" s="10" t="n"/>
-      <c r="I10" s="10" t="n"/>
-      <c r="J10" s="10" t="n"/>
-      <c r="K10" s="10" t="n"/>
     </row>
     <row r="11" ht="28" customHeight="1">
       <c r="A11" s="11" t="inlineStr">
@@ -964,7 +1027,7 @@
           <t>Requirement / ความต้องการ</t>
         </is>
       </c>
-      <c r="C11" s="12" t="n"/>
+      <c r="C11" s="61" t="n"/>
       <c r="D11" s="11" t="inlineStr">
         <is>
           <t>รองรับ
@@ -982,11 +1045,11 @@
           <t>Solutions / แนวทาง</t>
         </is>
       </c>
-      <c r="G11" s="12" t="n"/>
-      <c r="H11" s="12" t="n"/>
-      <c r="I11" s="12" t="n"/>
-      <c r="J11" s="12" t="n"/>
-      <c r="K11" s="12" t="n"/>
+      <c r="G11" s="62" t="n"/>
+      <c r="H11" s="62" t="n"/>
+      <c r="I11" s="62" t="n"/>
+      <c r="J11" s="62" t="n"/>
+      <c r="K11" s="61" t="n"/>
     </row>
     <row r="12" ht="22" customHeight="1">
       <c r="A12" s="13" t="n">
@@ -997,15 +1060,15 @@
           <t>(ระบุความต้องการของลูกค้า)</t>
         </is>
       </c>
-      <c r="C12" s="15" t="n"/>
+      <c r="C12" s="61" t="n"/>
       <c r="D12" s="15" t="n"/>
       <c r="E12" s="15" t="n"/>
       <c r="F12" s="15" t="n"/>
-      <c r="G12" s="15" t="n"/>
-      <c r="H12" s="15" t="n"/>
-      <c r="I12" s="15" t="n"/>
-      <c r="J12" s="15" t="n"/>
-      <c r="K12" s="15" t="n"/>
+      <c r="G12" s="62" t="n"/>
+      <c r="H12" s="62" t="n"/>
+      <c r="I12" s="62" t="n"/>
+      <c r="J12" s="62" t="n"/>
+      <c r="K12" s="61" t="n"/>
     </row>
     <row r="14" ht="22" customHeight="1">
       <c r="A14" s="9" t="inlineStr">
@@ -1013,16 +1076,6 @@
           <t xml:space="preserve">    🎁  Special Offers</t>
         </is>
       </c>
-      <c r="B14" s="10" t="n"/>
-      <c r="C14" s="10" t="n"/>
-      <c r="D14" s="10" t="n"/>
-      <c r="E14" s="10" t="n"/>
-      <c r="F14" s="10" t="n"/>
-      <c r="G14" s="10" t="n"/>
-      <c r="H14" s="10" t="n"/>
-      <c r="I14" s="10" t="n"/>
-      <c r="J14" s="10" t="n"/>
-      <c r="K14" s="10" t="n"/>
     </row>
     <row r="15" ht="20" customHeight="1">
       <c r="A15" s="11" t="inlineStr">
@@ -1035,19 +1088,19 @@
           <t>รายการ</t>
         </is>
       </c>
-      <c r="C15" s="12" t="n"/>
+      <c r="C15" s="61" t="n"/>
       <c r="D15" s="11" t="inlineStr">
         <is>
           <t>รายละเอียด</t>
         </is>
       </c>
-      <c r="E15" s="12" t="n"/>
-      <c r="F15" s="12" t="n"/>
-      <c r="G15" s="12" t="n"/>
-      <c r="H15" s="12" t="n"/>
-      <c r="I15" s="12" t="n"/>
-      <c r="J15" s="12" t="n"/>
-      <c r="K15" s="12" t="n"/>
+      <c r="E15" s="62" t="n"/>
+      <c r="F15" s="62" t="n"/>
+      <c r="G15" s="62" t="n"/>
+      <c r="H15" s="62" t="n"/>
+      <c r="I15" s="62" t="n"/>
+      <c r="J15" s="62" t="n"/>
+      <c r="K15" s="61" t="n"/>
     </row>
     <row r="16" ht="24" customHeight="1">
       <c r="A16" s="13" t="n">
@@ -1058,19 +1111,19 @@
           <t>ข้อเสนอพิเศษ</t>
         </is>
       </c>
-      <c r="C16" s="15" t="n"/>
+      <c r="C16" s="61" t="n"/>
       <c r="D16" s="17" t="inlineStr">
         <is>
           <t>สำหรับการสมัครใช้งานแพ็กเกจ (สัญญา 1 ปี) — 10 ฟรี 2 เมื่อชำระภายในเดือน</t>
         </is>
       </c>
-      <c r="E16" s="15" t="n"/>
-      <c r="F16" s="15" t="n"/>
-      <c r="G16" s="15" t="n"/>
-      <c r="H16" s="15" t="n"/>
-      <c r="I16" s="15" t="n"/>
-      <c r="J16" s="15" t="n"/>
-      <c r="K16" s="15" t="n"/>
+      <c r="E16" s="62" t="n"/>
+      <c r="F16" s="62" t="n"/>
+      <c r="G16" s="62" t="n"/>
+      <c r="H16" s="62" t="n"/>
+      <c r="I16" s="62" t="n"/>
+      <c r="J16" s="62" t="n"/>
+      <c r="K16" s="61" t="n"/>
     </row>
     <row r="17" ht="96" customHeight="1">
       <c r="A17" s="18" t="n">
@@ -1081,7 +1134,7 @@
           <t>บริการ</t>
         </is>
       </c>
-      <c r="C17" s="20" t="n"/>
+      <c r="C17" s="61" t="n"/>
       <c r="D17" s="21" t="inlineStr">
         <is>
           <t>• ไม่มีค่า MA
@@ -1092,13 +1145,13 @@
 • Training ฟรี 3 ครั้ง</t>
         </is>
       </c>
-      <c r="E17" s="20" t="n"/>
-      <c r="F17" s="20" t="n"/>
-      <c r="G17" s="20" t="n"/>
-      <c r="H17" s="20" t="n"/>
-      <c r="I17" s="20" t="n"/>
-      <c r="J17" s="20" t="n"/>
-      <c r="K17" s="20" t="n"/>
+      <c r="E17" s="62" t="n"/>
+      <c r="F17" s="62" t="n"/>
+      <c r="G17" s="62" t="n"/>
+      <c r="H17" s="62" t="n"/>
+      <c r="I17" s="62" t="n"/>
+      <c r="J17" s="62" t="n"/>
+      <c r="K17" s="61" t="n"/>
     </row>
     <row r="19" ht="22" customHeight="1">
       <c r="A19" s="9" t="inlineStr">
@@ -1106,16 +1159,6 @@
           <t xml:space="preserve">    📅  Timeline</t>
         </is>
       </c>
-      <c r="B19" s="10" t="n"/>
-      <c r="C19" s="10" t="n"/>
-      <c r="D19" s="10" t="n"/>
-      <c r="E19" s="10" t="n"/>
-      <c r="F19" s="10" t="n"/>
-      <c r="G19" s="10" t="n"/>
-      <c r="H19" s="10" t="n"/>
-      <c r="I19" s="10" t="n"/>
-      <c r="J19" s="10" t="n"/>
-      <c r="K19" s="10" t="n"/>
     </row>
     <row r="20" ht="16" customHeight="1">
       <c r="A20" s="22" t="inlineStr">
@@ -1130,7 +1173,7 @@
           <t>Step</t>
         </is>
       </c>
-      <c r="B21" s="24" t="n"/>
+      <c r="B21" s="63" t="n"/>
       <c r="C21" s="11" t="inlineStr">
         <is>
           <t>รายการ</t>
@@ -1141,22 +1184,22 @@
           <t>Month 1</t>
         </is>
       </c>
-      <c r="E21" s="24" t="n"/>
-      <c r="F21" s="24" t="n"/>
-      <c r="G21" s="24" t="n"/>
+      <c r="E21" s="62" t="n"/>
+      <c r="F21" s="62" t="n"/>
+      <c r="G21" s="61" t="n"/>
       <c r="H21" s="25" t="inlineStr">
         <is>
           <t>Month 2</t>
         </is>
       </c>
-      <c r="I21" s="24" t="n"/>
-      <c r="J21" s="24" t="n"/>
-      <c r="K21" s="24" t="n"/>
+      <c r="I21" s="62" t="n"/>
+      <c r="J21" s="62" t="n"/>
+      <c r="K21" s="61" t="n"/>
     </row>
     <row r="22" ht="16" customHeight="1">
-      <c r="A22" s="24" t="n"/>
-      <c r="B22" s="24" t="n"/>
-      <c r="C22" s="24" t="n"/>
+      <c r="A22" s="64" t="n"/>
+      <c r="B22" s="65" t="n"/>
+      <c r="C22" s="66" t="n"/>
       <c r="D22" s="26" t="inlineStr">
         <is>
           <t>W1</t>
@@ -1232,8 +1275,8 @@
       <c r="K23" s="15" t="n"/>
     </row>
     <row r="24" ht="22" customHeight="1">
-      <c r="A24" s="24" t="n"/>
-      <c r="B24" s="24" t="n"/>
+      <c r="A24" s="67" t="n"/>
+      <c r="B24" s="67" t="n"/>
       <c r="C24" s="29" t="inlineStr">
         <is>
           <t>พิจารณา / Consider</t>
@@ -1257,8 +1300,8 @@
       <c r="K24" s="15" t="n"/>
     </row>
     <row r="25" ht="22" customHeight="1">
-      <c r="A25" s="24" t="n"/>
-      <c r="B25" s="24" t="n"/>
+      <c r="A25" s="66" t="n"/>
+      <c r="B25" s="66" t="n"/>
       <c r="C25" s="29" t="inlineStr">
         <is>
           <t>ชำระเงิน / Paid</t>
@@ -1311,8 +1354,8 @@
       <c r="K26" s="15" t="n"/>
     </row>
     <row r="27" ht="22" customHeight="1">
-      <c r="A27" s="24" t="n"/>
-      <c r="B27" s="24" t="n"/>
+      <c r="A27" s="67" t="n"/>
+      <c r="B27" s="67" t="n"/>
       <c r="C27" s="29" t="inlineStr">
         <is>
           <t>นำเข้าข้อมูลพนักงาน</t>
@@ -1332,8 +1375,8 @@
       <c r="K27" s="15" t="n"/>
     </row>
     <row r="28" ht="22" customHeight="1">
-      <c r="A28" s="24" t="n"/>
-      <c r="B28" s="24" t="n"/>
+      <c r="A28" s="67" t="n"/>
+      <c r="B28" s="67" t="n"/>
       <c r="C28" s="29" t="inlineStr">
         <is>
           <t>การ Setting ระบบ</t>
@@ -1353,8 +1396,8 @@
       <c r="K28" s="15" t="n"/>
     </row>
     <row r="29" ht="22" customHeight="1">
-      <c r="A29" s="24" t="n"/>
-      <c r="B29" s="24" t="n"/>
+      <c r="A29" s="67" t="n"/>
+      <c r="B29" s="67" t="n"/>
       <c r="C29" s="29" t="inlineStr">
         <is>
           <t>Online Training 3 ครั้ง</t>
@@ -1378,8 +1421,8 @@
       </c>
     </row>
     <row r="30" ht="22" customHeight="1">
-      <c r="A30" s="24" t="n"/>
-      <c r="B30" s="24" t="n"/>
+      <c r="A30" s="67" t="n"/>
+      <c r="B30" s="67" t="n"/>
       <c r="C30" s="29" t="inlineStr">
         <is>
           <t>ทดสอบทำเงินเดือน</t>
@@ -1399,8 +1442,8 @@
       <c r="K30" s="15" t="n"/>
     </row>
     <row r="31" ht="22" customHeight="1">
-      <c r="A31" s="24" t="n"/>
-      <c r="B31" s="24" t="n"/>
+      <c r="A31" s="67" t="n"/>
+      <c r="B31" s="67" t="n"/>
       <c r="C31" s="29" t="inlineStr">
         <is>
           <t>การเตรียมนำเข้าข้อมูลย้อนหลัง</t>
@@ -1420,8 +1463,8 @@
       <c r="K31" s="15" t="n"/>
     </row>
     <row r="32" ht="22" customHeight="1">
-      <c r="A32" s="24" t="n"/>
-      <c r="B32" s="24" t="n"/>
+      <c r="A32" s="66" t="n"/>
+      <c r="B32" s="66" t="n"/>
       <c r="C32" s="29" t="inlineStr">
         <is>
           <t>การนำเข้าข้อมูลย้อนหลัง / Go live</t>
@@ -1506,11 +1549,6 @@
           <t>💰  ราคา &amp; แพ็กเกจ</t>
         </is>
       </c>
-      <c r="B2" s="10" t="n"/>
-      <c r="C2" s="10" t="n"/>
-      <c r="D2" s="10" t="n"/>
-      <c r="E2" s="10" t="n"/>
-      <c r="F2" s="10" t="n"/>
       <c r="G2" s="36" t="inlineStr">
         <is>
           <t>Human</t>
@@ -1563,7 +1601,7 @@
           <t>ราคาปกติ (ไม่มีโปร / ราย 1 ปี)</t>
         </is>
       </c>
-      <c r="C7" s="15" t="n"/>
+      <c r="C7" s="61" t="n"/>
       <c r="D7" s="13" t="inlineStr">
         <is>
           <t>—</t>
@@ -1579,7 +1617,7 @@
           <t>จ่าย 10 ฟรี 2 เดือน</t>
         </is>
       </c>
-      <c r="C8" s="20" t="n"/>
+      <c r="C8" s="61" t="n"/>
       <c r="D8" s="18" t="inlineStr">
         <is>
           <t>—</t>
@@ -1595,7 +1633,7 @@
           <t>💎 ยอดสุทธิ</t>
         </is>
       </c>
-      <c r="C9" s="15" t="n"/>
+      <c r="C9" s="61" t="n"/>
       <c r="D9" s="44" t="inlineStr">
         <is>
           <t>—</t>
@@ -1611,7 +1649,7 @@
           <t>ราคาเฉลี่ยต่อเดือน</t>
         </is>
       </c>
-      <c r="C10" s="20" t="n"/>
+      <c r="C10" s="61" t="n"/>
       <c r="D10" s="18" t="inlineStr">
         <is>
           <t>—</t>
@@ -1663,8 +1701,6 @@
           <t>✅  Features ที่ต้องการใช้งาน</t>
         </is>
       </c>
-      <c r="B2" s="10" t="n"/>
-      <c r="C2" s="10" t="n"/>
       <c r="D2" s="46" t="inlineStr">
         <is>
           <t>Soft</t>
@@ -1697,9 +1733,6 @@
           <t xml:space="preserve">  Channel</t>
         </is>
       </c>
-      <c r="B6" s="10" t="n"/>
-      <c r="C6" s="10" t="n"/>
-      <c r="D6" s="10" t="n"/>
     </row>
     <row r="7" ht="17" customHeight="1">
       <c r="A7" s="15" t="n"/>
@@ -1713,7 +1746,7 @@
           <t>Web Browser</t>
         </is>
       </c>
-      <c r="D7" s="15" t="n"/>
+      <c r="D7" s="61" t="n"/>
     </row>
     <row r="8" ht="17" customHeight="1">
       <c r="A8" s="20" t="n"/>
@@ -1727,7 +1760,7 @@
           <t>Mobile Application / Line OA</t>
         </is>
       </c>
-      <c r="D8" s="20" t="n"/>
+      <c r="D8" s="61" t="n"/>
     </row>
     <row r="9" ht="18" customHeight="1">
       <c r="A9" s="49" t="inlineStr">
@@ -1735,9 +1768,6 @@
           <t xml:space="preserve">  โครงสร้างทั่วไป</t>
         </is>
       </c>
-      <c r="B9" s="10" t="n"/>
-      <c r="C9" s="10" t="n"/>
-      <c r="D9" s="10" t="n"/>
     </row>
     <row r="10" ht="17" customHeight="1">
       <c r="A10" s="15" t="n"/>
@@ -1751,7 +1781,7 @@
           <t>รองรับหลายนิติบุคคล</t>
         </is>
       </c>
-      <c r="D10" s="15" t="n"/>
+      <c r="D10" s="61" t="n"/>
     </row>
     <row r="11" ht="17" customHeight="1">
       <c r="A11" s="20" t="n"/>
@@ -1765,7 +1795,7 @@
           <t>รองรับหลายสาขา</t>
         </is>
       </c>
-      <c r="D11" s="20" t="n"/>
+      <c r="D11" s="61" t="n"/>
     </row>
     <row r="12" ht="17" customHeight="1">
       <c r="A12" s="15" t="n"/>
@@ -1779,7 +1809,7 @@
           <t>รองรับ 3 ภาษา (ไทย/อังกฤษ/พม่า)</t>
         </is>
       </c>
-      <c r="D12" s="15" t="n"/>
+      <c r="D12" s="61" t="n"/>
     </row>
     <row r="13" ht="18" customHeight="1">
       <c r="A13" s="49" t="inlineStr">
@@ -1787,9 +1817,6 @@
           <t xml:space="preserve">  โครงสร้างองค์กร</t>
         </is>
       </c>
-      <c r="B13" s="10" t="n"/>
-      <c r="C13" s="10" t="n"/>
-      <c r="D13" s="10" t="n"/>
     </row>
     <row r="14" ht="17" customHeight="1">
       <c r="A14" s="15" t="n"/>
@@ -1803,7 +1830,7 @@
           <t>โครงสร้างองค์กร / โครงสร้างตำแหน่ง</t>
         </is>
       </c>
-      <c r="D14" s="15" t="n"/>
+      <c r="D14" s="61" t="n"/>
     </row>
     <row r="15" ht="17" customHeight="1">
       <c r="A15" s="20" t="n"/>
@@ -1817,7 +1844,7 @@
           <t>เก็บประวัติข้อมูลพนักงาน</t>
         </is>
       </c>
-      <c r="D15" s="20" t="n"/>
+      <c r="D15" s="61" t="n"/>
     </row>
     <row r="16" ht="17" customHeight="1">
       <c r="A16" s="15" t="n"/>
@@ -1831,7 +1858,7 @@
           <t>รองรับการเก็บไฟล์ไม่จำกัดพื้นที่</t>
         </is>
       </c>
-      <c r="D16" s="15" t="n"/>
+      <c r="D16" s="61" t="n"/>
     </row>
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="49" t="inlineStr">
@@ -1839,9 +1866,6 @@
           <t xml:space="preserve">  จัดการสิทธิ์การเข้าถึงข้อมูล</t>
         </is>
       </c>
-      <c r="B17" s="10" t="n"/>
-      <c r="C17" s="10" t="n"/>
-      <c r="D17" s="10" t="n"/>
     </row>
     <row r="18" ht="17" customHeight="1">
       <c r="A18" s="15" t="n"/>
@@ -1855,7 +1879,7 @@
           <t>กำหนดสิทธิ์ผู้ดูแลระบบ (ไม่จำกัด User)</t>
         </is>
       </c>
-      <c r="D18" s="15" t="n"/>
+      <c r="D18" s="61" t="n"/>
     </row>
     <row r="19" ht="17" customHeight="1">
       <c r="A19" s="20" t="n"/>
@@ -1869,7 +1893,7 @@
           <t>กำหนดสิทธิ์มองเห็น/แก้ไขของแต่ละ User</t>
         </is>
       </c>
-      <c r="D19" s="20" t="n"/>
+      <c r="D19" s="61" t="n"/>
     </row>
     <row r="20" ht="17" customHeight="1">
       <c r="A20" s="15" t="n"/>
@@ -1883,7 +1907,7 @@
           <t>จัดกลุ่มผู้ใช้ได้</t>
         </is>
       </c>
-      <c r="D20" s="15" t="n"/>
+      <c r="D20" s="61" t="n"/>
     </row>
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="49" t="inlineStr">
@@ -1891,9 +1915,6 @@
           <t xml:space="preserve">  ระบบความปลอดภัย</t>
         </is>
       </c>
-      <c r="B21" s="10" t="n"/>
-      <c r="C21" s="10" t="n"/>
-      <c r="D21" s="10" t="n"/>
     </row>
     <row r="22" ht="17" customHeight="1">
       <c r="A22" s="15" t="n"/>
@@ -1907,7 +1928,7 @@
           <t>Strong Password</t>
         </is>
       </c>
-      <c r="D22" s="15" t="n"/>
+      <c r="D22" s="61" t="n"/>
     </row>
     <row r="23" ht="17" customHeight="1">
       <c r="A23" s="20" t="n"/>
@@ -1921,7 +1942,7 @@
           <t>PDPA Conceal</t>
         </is>
       </c>
-      <c r="D23" s="20" t="n"/>
+      <c r="D23" s="61" t="n"/>
     </row>
     <row r="24" ht="18" customHeight="1">
       <c r="A24" s="49" t="inlineStr">
@@ -1929,9 +1950,6 @@
           <t xml:space="preserve">  จัดการกะ</t>
         </is>
       </c>
-      <c r="B24" s="10" t="n"/>
-      <c r="C24" s="10" t="n"/>
-      <c r="D24" s="10" t="n"/>
     </row>
     <row r="25" ht="17" customHeight="1">
       <c r="A25" s="15" t="n"/>
@@ -1945,7 +1963,7 @@
           <t>กะได้หลายรูปแบบ (Default / หลายกะ / Excel Import)</t>
         </is>
       </c>
-      <c r="D25" s="15" t="n"/>
+      <c r="D25" s="61" t="n"/>
     </row>
     <row r="26" ht="17" customHeight="1">
       <c r="A26" s="20" t="n"/>
@@ -1959,7 +1977,7 @@
           <t>วางแผนกะรายเดือน / รายสัปดาห์</t>
         </is>
       </c>
-      <c r="D26" s="20" t="n"/>
+      <c r="D26" s="61" t="n"/>
     </row>
     <row r="27" ht="17" customHeight="1">
       <c r="A27" s="15" t="n"/>
@@ -1973,7 +1991,7 @@
           <t>สิทธิ์จัดกะแบบยืดหยุ่น (HR / หัวหน้า / พนักงาน)</t>
         </is>
       </c>
-      <c r="D27" s="15" t="n"/>
+      <c r="D27" s="61" t="n"/>
     </row>
     <row r="28" ht="18" customHeight="1">
       <c r="A28" s="49" t="inlineStr">
@@ -1981,9 +1999,6 @@
           <t xml:space="preserve">  ลงเวลาการทำงาน</t>
         </is>
       </c>
-      <c r="B28" s="10" t="n"/>
-      <c r="C28" s="10" t="n"/>
-      <c r="D28" s="10" t="n"/>
     </row>
     <row r="29" ht="17" customHeight="1">
       <c r="A29" s="15" t="n"/>
@@ -1997,7 +2012,7 @@
           <t>Face Scan (Face Recognition)</t>
         </is>
       </c>
-      <c r="D29" s="15" t="n"/>
+      <c r="D29" s="61" t="n"/>
     </row>
     <row r="30" ht="17" customHeight="1">
       <c r="A30" s="20" t="n"/>
@@ -2011,7 +2026,7 @@
           <t>GPS</t>
         </is>
       </c>
-      <c r="D30" s="20" t="n"/>
+      <c r="D30" s="61" t="n"/>
     </row>
     <row r="31" ht="17" customHeight="1">
       <c r="A31" s="15" t="n"/>
@@ -2025,7 +2040,7 @@
           <t>เครื่องสแกนนิ้ว</t>
         </is>
       </c>
-      <c r="D31" s="15" t="n"/>
+      <c r="D31" s="61" t="n"/>
     </row>
     <row r="32" ht="18" customHeight="1">
       <c r="A32" s="49" t="inlineStr">
@@ -2033,9 +2048,6 @@
           <t xml:space="preserve">  เอกสารและการอนุมัติ</t>
         </is>
       </c>
-      <c r="B32" s="10" t="n"/>
-      <c r="C32" s="10" t="n"/>
-      <c r="D32" s="10" t="n"/>
     </row>
     <row r="33" ht="17" customHeight="1">
       <c r="A33" s="15" t="n"/>
@@ -2049,7 +2061,7 @@
           <t>เอกสารพื้นฐาน (ลา / OT / สลับกะ / ขอเพิ่มเวลา)</t>
         </is>
       </c>
-      <c r="D33" s="15" t="n"/>
+      <c r="D33" s="61" t="n"/>
     </row>
     <row r="34" ht="17" customHeight="1">
       <c r="A34" s="20" t="n"/>
@@ -2063,7 +2075,7 @@
           <t>เบิกเงินล่วงหน้า</t>
         </is>
       </c>
-      <c r="D34" s="20" t="n"/>
+      <c r="D34" s="61" t="n"/>
     </row>
     <row r="35" ht="17" customHeight="1">
       <c r="A35" s="15" t="n"/>
@@ -2077,7 +2089,7 @@
           <t>หนังสือรับรองเงินเดือน</t>
         </is>
       </c>
-      <c r="D35" s="15" t="n"/>
+      <c r="D35" s="61" t="n"/>
     </row>
     <row r="36" ht="17" customHeight="1">
       <c r="A36" s="20" t="n"/>
@@ -2091,7 +2103,7 @@
           <t>อนุมัติผ่าน Website</t>
         </is>
       </c>
-      <c r="D36" s="20" t="n"/>
+      <c r="D36" s="61" t="n"/>
     </row>
     <row r="37" ht="17" customHeight="1">
       <c r="A37" s="15" t="n"/>
@@ -2105,7 +2117,7 @@
           <t>อนุมัติผ่าน App</t>
         </is>
       </c>
-      <c r="D37" s="15" t="n"/>
+      <c r="D37" s="61" t="n"/>
     </row>
     <row r="38" ht="17" customHeight="1">
       <c r="A38" s="20" t="n"/>
@@ -2119,7 +2131,7 @@
           <t>สายการอนุมัติ 3-5 ขั้น</t>
         </is>
       </c>
-      <c r="D38" s="20" t="n"/>
+      <c r="D38" s="61" t="n"/>
     </row>
     <row r="39" ht="18" customHeight="1">
       <c r="A39" s="49" t="inlineStr">
@@ -2127,9 +2139,6 @@
           <t xml:space="preserve">  การคำนวณเงินเดือน</t>
         </is>
       </c>
-      <c r="B39" s="10" t="n"/>
-      <c r="C39" s="10" t="n"/>
-      <c r="D39" s="10" t="n"/>
     </row>
     <row r="40" ht="17" customHeight="1">
       <c r="A40" s="15" t="n"/>
@@ -2143,7 +2152,7 @@
           <t>รายรับ/รายจ่าย (อัตโนมัติ / Manual)</t>
         </is>
       </c>
-      <c r="D40" s="15" t="n"/>
+      <c r="D40" s="61" t="n"/>
     </row>
     <row r="41" ht="17" customHeight="1">
       <c r="A41" s="20" t="n"/>
@@ -2157,7 +2166,7 @@
           <t>งวดเงินเดือน สูงสุด 4 งวด</t>
         </is>
       </c>
-      <c r="D41" s="20" t="n"/>
+      <c r="D41" s="61" t="n"/>
     </row>
     <row r="42" ht="17" customHeight="1">
       <c r="A42" s="15" t="n"/>
@@ -2171,7 +2180,7 @@
           <t>สลิปเงินเดือน</t>
         </is>
       </c>
-      <c r="D42" s="15" t="n"/>
+      <c r="D42" s="61" t="n"/>
     </row>
     <row r="43" ht="17" customHeight="1">
       <c r="A43" s="20" t="n"/>
@@ -2185,7 +2194,7 @@
           <t>Text File นำส่งธนาคาร</t>
         </is>
       </c>
-      <c r="D43" s="20" t="n"/>
+      <c r="D43" s="61" t="n"/>
     </row>
     <row r="44" ht="17" customHeight="1">
       <c r="A44" s="15" t="n"/>
@@ -2199,7 +2208,7 @@
           <t>ภาษี / ประกันสังคม / กองทุน</t>
         </is>
       </c>
-      <c r="D44" s="15" t="n"/>
+      <c r="D44" s="61" t="n"/>
     </row>
     <row r="45" ht="17" customHeight="1">
       <c r="A45" s="20" t="n"/>
@@ -2213,7 +2222,7 @@
           <t>เบี้ยเลี้ยง / เบี้ยขยัน</t>
         </is>
       </c>
-      <c r="D45" s="20" t="n"/>
+      <c r="D45" s="61" t="n"/>
     </row>
     <row r="46" ht="18" customHeight="1">
       <c r="A46" s="49" t="inlineStr">
@@ -2221,9 +2230,6 @@
           <t xml:space="preserve">  รายงาน</t>
         </is>
       </c>
-      <c r="B46" s="10" t="n"/>
-      <c r="C46" s="10" t="n"/>
-      <c r="D46" s="10" t="n"/>
     </row>
     <row r="47" ht="17" customHeight="1">
       <c r="A47" s="15" t="n"/>
@@ -2237,7 +2243,7 @@
           <t>รายงานมากกว่า 50 แบบ (.pdf / .xlsx / .txt / .dat)</t>
         </is>
       </c>
-      <c r="D47" s="15" t="n"/>
+      <c r="D47" s="61" t="n"/>
     </row>
     <row r="48" ht="18" customHeight="1">
       <c r="A48" s="49" t="inlineStr">
@@ -2245,9 +2251,6 @@
           <t xml:space="preserve">  การเรียนรู้และพัฒนาองค์กร (HRD)</t>
         </is>
       </c>
-      <c r="B48" s="10" t="n"/>
-      <c r="C48" s="10" t="n"/>
-      <c r="D48" s="10" t="n"/>
     </row>
     <row r="49" ht="17" customHeight="1">
       <c r="A49" s="15" t="n"/>
@@ -2261,7 +2264,7 @@
           <t>E-Library / E-Learning</t>
         </is>
       </c>
-      <c r="D49" s="15" t="n"/>
+      <c r="D49" s="61" t="n"/>
     </row>
     <row r="50" ht="17" customHeight="1">
       <c r="A50" s="20" t="n"/>
@@ -2275,7 +2278,7 @@
           <t>ประเมินพนักงาน (ไม่จำกัดรอบ)</t>
         </is>
       </c>
-      <c r="D50" s="20" t="n"/>
+      <c r="D50" s="61" t="n"/>
     </row>
     <row r="51" ht="17" customHeight="1">
       <c r="A51" s="15" t="n"/>
@@ -2289,7 +2292,7 @@
           <t>KPI Profile</t>
         </is>
       </c>
-      <c r="D51" s="15" t="n"/>
+      <c r="D51" s="61" t="n"/>
     </row>
     <row r="52" ht="17" customHeight="1">
       <c r="A52" s="20" t="n"/>
@@ -2303,7 +2306,7 @@
           <t>บันทึกการฝึกอบรม</t>
         </is>
       </c>
-      <c r="D52" s="20" t="n"/>
+      <c r="D52" s="61" t="n"/>
     </row>
     <row r="53" ht="18" customHeight="1">
       <c r="A53" s="49" t="inlineStr">
@@ -2311,9 +2314,6 @@
           <t xml:space="preserve">  ระบบรับสมัครพนักงาน</t>
         </is>
       </c>
-      <c r="B53" s="10" t="n"/>
-      <c r="C53" s="10" t="n"/>
-      <c r="D53" s="10" t="n"/>
     </row>
     <row r="54" ht="17" customHeight="1">
       <c r="A54" s="15" t="n"/>
@@ -2327,7 +2327,7 @@
           <t>ใบสมัครงานออนไลน์</t>
         </is>
       </c>
-      <c r="D54" s="15" t="n"/>
+      <c r="D54" s="61" t="n"/>
     </row>
     <row r="55" ht="17" customHeight="1">
       <c r="A55" s="20" t="n"/>
@@ -2341,7 +2341,7 @@
           <t>ระบบติดตามผู้สมัคร</t>
         </is>
       </c>
-      <c r="D55" s="20" t="n"/>
+      <c r="D55" s="61" t="n"/>
     </row>
     <row r="56" ht="17" customHeight="1">
       <c r="A56" s="15" t="n"/>
@@ -2355,7 +2355,7 @@
           <t>เอกสารสัญญาจ้าง (ทดลองงาน/บรรจุ)</t>
         </is>
       </c>
-      <c r="D56" s="15" t="n"/>
+      <c r="D56" s="61" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="54">
@@ -2448,16 +2448,6 @@
           <t xml:space="preserve">    📅  Timeline</t>
         </is>
       </c>
-      <c r="B1" s="10" t="n"/>
-      <c r="C1" s="10" t="n"/>
-      <c r="D1" s="10" t="n"/>
-      <c r="E1" s="10" t="n"/>
-      <c r="F1" s="10" t="n"/>
-      <c r="G1" s="10" t="n"/>
-      <c r="H1" s="10" t="n"/>
-      <c r="I1" s="10" t="n"/>
-      <c r="J1" s="10" t="n"/>
-      <c r="K1" s="10" t="n"/>
     </row>
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="22" t="inlineStr">
@@ -2487,22 +2477,22 @@
           <t>Month 1</t>
         </is>
       </c>
-      <c r="E3" s="51" t="n"/>
-      <c r="F3" s="51" t="n"/>
-      <c r="G3" s="51" t="n"/>
+      <c r="E3" s="62" t="n"/>
+      <c r="F3" s="62" t="n"/>
+      <c r="G3" s="61" t="n"/>
       <c r="H3" s="25" t="inlineStr">
         <is>
           <t>Month 2</t>
         </is>
       </c>
-      <c r="I3" s="51" t="n"/>
-      <c r="J3" s="51" t="n"/>
-      <c r="K3" s="51" t="n"/>
+      <c r="I3" s="62" t="n"/>
+      <c r="J3" s="62" t="n"/>
+      <c r="K3" s="61" t="n"/>
     </row>
     <row r="4" ht="16" customHeight="1">
-      <c r="A4" s="24" t="n"/>
-      <c r="B4" s="24" t="n"/>
-      <c r="C4" s="24" t="n"/>
+      <c r="A4" s="66" t="n"/>
+      <c r="B4" s="66" t="n"/>
+      <c r="C4" s="66" t="n"/>
       <c r="D4" s="26" t="inlineStr">
         <is>
           <t>W1</t>
@@ -2600,16 +2590,16 @@
           <t>●  การเตรียมข้อมูลสำหรับขึ้นระบบ</t>
         </is>
       </c>
-      <c r="B7" s="24" t="n"/>
-      <c r="C7" s="24" t="n"/>
-      <c r="D7" s="24" t="n"/>
-      <c r="E7" s="24" t="n"/>
-      <c r="F7" s="24" t="n"/>
-      <c r="G7" s="24" t="n"/>
-      <c r="H7" s="24" t="n"/>
-      <c r="I7" s="24" t="n"/>
-      <c r="J7" s="24" t="n"/>
-      <c r="K7" s="24" t="n"/>
+      <c r="B7" s="62" t="n"/>
+      <c r="C7" s="62" t="n"/>
+      <c r="D7" s="62" t="n"/>
+      <c r="E7" s="62" t="n"/>
+      <c r="F7" s="62" t="n"/>
+      <c r="G7" s="62" t="n"/>
+      <c r="H7" s="62" t="n"/>
+      <c r="I7" s="62" t="n"/>
+      <c r="J7" s="62" t="n"/>
+      <c r="K7" s="61" t="n"/>
     </row>
     <row r="8" ht="18" customHeight="1">
       <c r="A8" s="40" t="n">
@@ -2755,16 +2745,16 @@
           <t>●  นัดการสอนใช้งาน Application / Website</t>
         </is>
       </c>
-      <c r="B14" s="24" t="n"/>
-      <c r="C14" s="24" t="n"/>
-      <c r="D14" s="24" t="n"/>
-      <c r="E14" s="24" t="n"/>
-      <c r="F14" s="24" t="n"/>
-      <c r="G14" s="24" t="n"/>
-      <c r="H14" s="24" t="n"/>
-      <c r="I14" s="24" t="n"/>
-      <c r="J14" s="24" t="n"/>
-      <c r="K14" s="24" t="n"/>
+      <c r="B14" s="62" t="n"/>
+      <c r="C14" s="62" t="n"/>
+      <c r="D14" s="62" t="n"/>
+      <c r="E14" s="62" t="n"/>
+      <c r="F14" s="62" t="n"/>
+      <c r="G14" s="62" t="n"/>
+      <c r="H14" s="62" t="n"/>
+      <c r="I14" s="62" t="n"/>
+      <c r="J14" s="62" t="n"/>
+      <c r="K14" s="61" t="n"/>
     </row>
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="40" t="n">
@@ -2795,16 +2785,16 @@
           <t>●  Internal Training (ด้วยตัวเอง)</t>
         </is>
       </c>
-      <c r="B16" s="24" t="n"/>
-      <c r="C16" s="24" t="n"/>
-      <c r="D16" s="24" t="n"/>
-      <c r="E16" s="24" t="n"/>
-      <c r="F16" s="24" t="n"/>
-      <c r="G16" s="24" t="n"/>
-      <c r="H16" s="24" t="n"/>
-      <c r="I16" s="24" t="n"/>
-      <c r="J16" s="24" t="n"/>
-      <c r="K16" s="24" t="n"/>
+      <c r="B16" s="62" t="n"/>
+      <c r="C16" s="62" t="n"/>
+      <c r="D16" s="62" t="n"/>
+      <c r="E16" s="62" t="n"/>
+      <c r="F16" s="62" t="n"/>
+      <c r="G16" s="62" t="n"/>
+      <c r="H16" s="62" t="n"/>
+      <c r="I16" s="62" t="n"/>
+      <c r="J16" s="62" t="n"/>
+      <c r="K16" s="61" t="n"/>
     </row>
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="40" t="n">
@@ -2835,16 +2825,16 @@
           <t>●  เริ่มการใช้งาน (Parallel Run)</t>
         </is>
       </c>
-      <c r="B18" s="24" t="n"/>
-      <c r="C18" s="24" t="n"/>
-      <c r="D18" s="24" t="n"/>
-      <c r="E18" s="24" t="n"/>
-      <c r="F18" s="24" t="n"/>
-      <c r="G18" s="24" t="n"/>
-      <c r="H18" s="24" t="n"/>
-      <c r="I18" s="24" t="n"/>
-      <c r="J18" s="24" t="n"/>
-      <c r="K18" s="24" t="n"/>
+      <c r="B18" s="62" t="n"/>
+      <c r="C18" s="62" t="n"/>
+      <c r="D18" s="62" t="n"/>
+      <c r="E18" s="62" t="n"/>
+      <c r="F18" s="62" t="n"/>
+      <c r="G18" s="62" t="n"/>
+      <c r="H18" s="62" t="n"/>
+      <c r="I18" s="62" t="n"/>
+      <c r="J18" s="62" t="n"/>
+      <c r="K18" s="61" t="n"/>
     </row>
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="40" t="n">
@@ -2940,16 +2930,16 @@
           <t>●  เตรียมข้อมูลเงินเดือน (ย้อนหลัง)</t>
         </is>
       </c>
-      <c r="B23" s="24" t="n"/>
-      <c r="C23" s="24" t="n"/>
-      <c r="D23" s="24" t="n"/>
-      <c r="E23" s="24" t="n"/>
-      <c r="F23" s="24" t="n"/>
-      <c r="G23" s="24" t="n"/>
-      <c r="H23" s="24" t="n"/>
-      <c r="I23" s="24" t="n"/>
-      <c r="J23" s="24" t="n"/>
-      <c r="K23" s="24" t="n"/>
+      <c r="B23" s="62" t="n"/>
+      <c r="C23" s="62" t="n"/>
+      <c r="D23" s="62" t="n"/>
+      <c r="E23" s="62" t="n"/>
+      <c r="F23" s="62" t="n"/>
+      <c r="G23" s="62" t="n"/>
+      <c r="H23" s="62" t="n"/>
+      <c r="I23" s="62" t="n"/>
+      <c r="J23" s="62" t="n"/>
+      <c r="K23" s="61" t="n"/>
     </row>
     <row r="24" ht="18" customHeight="1">
       <c r="A24" s="40" t="n">

</xml_diff>

<commit_message>
Apply Anuphan font and re-add styled Requirement Tracker sheet
- All sheets switched to Anuphan font
- Re-added Requirement Tracker sheet (web-matched colors: blue header, filled Type/Status badges) before Timeline
</commit_message>
<xml_diff>
--- a/Customer_Requirement_Report.xlsx
+++ b/Customer_Requirement_Report.xlsx
@@ -10,7 +10,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Price" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Features" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirement Tracker" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="30">
+  <fonts count="67">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -191,8 +192,217 @@
       <color rgb="00374151"/>
       <sz val="9"/>
     </font>
+    <font>
+      <name val="Anuphan"/>
+      <color theme="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Anuphan"/>
+      <b val="1"/>
+      <color rgb="001A56DB"/>
+      <sz val="20"/>
+    </font>
+    <font>
+      <name val="Anuphan"/>
+      <b val="1"/>
+      <color rgb="00F47B20"/>
+      <sz val="15"/>
+    </font>
+    <font>
+      <name val="Anuphan"/>
+      <b val="1"/>
+      <color rgb="00F47B20"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Anuphan"/>
+      <color rgb="009CA3AF"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Anuphan"/>
+      <color rgb="009CA3AF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Anuphan"/>
+      <b val="1"/>
+      <color rgb="001A56DB"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Anuphan"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Anuphan"/>
+      <b val="1"/>
+      <color rgb="001E3A8A"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Anuphan"/>
+      <b val="1"/>
+      <color rgb="00111827"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Anuphan"/>
+      <color rgb="00374151"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Anuphan"/>
+      <color rgb="00374151"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Anuphan"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Anuphan"/>
+      <b val="1"/>
+      <color rgb="001E3A8A"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Anuphan"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="Anuphan"/>
+      <b val="1"/>
+      <color rgb="001A56DB"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Anuphan"/>
+      <b val="1"/>
+      <color rgb="00111827"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Anuphan"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="Anuphan"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Anuphan"/>
+      <color rgb="001E3A8A"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Anuphan"/>
+      <color rgb="001E3A8A"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Anuphan"/>
+      <b val="1"/>
+      <color rgb="00065F46"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Anuphan"/>
+      <color rgb="00065F46"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Anuphan"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Anuphan"/>
+      <color rgb="00065F46"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Anuphan"/>
+      <b val="1"/>
+      <color rgb="005B21B6"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Anuphan"/>
+      <b val="1"/>
+      <color rgb="00065F46"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Anuphan"/>
+      <b val="1"/>
+      <color rgb="001A56DB"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Anuphan"/>
+      <b val="1"/>
+      <color rgb="001E40AF"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Anuphan"/>
+      <b val="1"/>
+      <color rgb="00374151"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Anuphan"/>
+      <color rgb="00374151"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Anuphan"/>
+      <b val="1"/>
+      <color rgb="006B7280"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Anuphan"/>
+      <b val="1"/>
+      <color rgb="001240B0"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Anuphan"/>
+      <b val="1"/>
+      <color rgb="00C85E0F"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Anuphan"/>
+      <b val="1"/>
+      <color rgb="001240B0"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Anuphan"/>
+      <b val="1"/>
+      <color rgb="00991B1B"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Anuphan"/>
+      <b val="1"/>
+      <color rgb="00065F46"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="15">
+  <fills count="17">
     <fill>
       <patternFill/>
     </fill>
@@ -264,8 +474,18 @@
         <fgColor rgb="0016A34A"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0078350F"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FEE2E2"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="12">
+  <borders count="14">
     <border>
       <left/>
       <right/>
@@ -395,11 +615,39 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="001240B0"/>
+      </left>
+      <right style="thin">
+        <color rgb="001240B0"/>
+      </right>
+      <top style="thin">
+        <color rgb="001240B0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="001240B0"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00D1D5DB"/>
+      </left>
+      <right style="thin">
+        <color rgb="00D1D5DB"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D1D5DB"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D1D5DB"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="68">
+  <cellXfs count="147">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -566,6 +814,213 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="35" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="39" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="40" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="40" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="42" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="42" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="43" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="44" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="45" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="46" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="37" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="30" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="30" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="47" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="48" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="48" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="49" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="50" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="34" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="40" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="40" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="51" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="52" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="48" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="49" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="49" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="53" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="54" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="37" fillId="4" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="61" fillId="6" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="60" fillId="6" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="42" fillId="4" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="62" fillId="6" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="63" fillId="2" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="61" fillId="5" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="60" fillId="5" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="42" fillId="15" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="62" fillId="5" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="64" fillId="3" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="42" fillId="12" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="65" fillId="16" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="42" fillId="14" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="66" fillId="10" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="55" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="42" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="56" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="46" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="57" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="58" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="59" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="59" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="42" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -931,7 +1386,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A2:K32"/>
+  <dimension ref="A1:K32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -947,195 +1402,323 @@
     <col width="6" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
+    <row r="1">
+      <c r="A1" s="68" t="n"/>
+      <c r="B1" s="68" t="n"/>
+      <c r="C1" s="68" t="n"/>
+      <c r="D1" s="68" t="n"/>
+      <c r="E1" s="68" t="n"/>
+      <c r="F1" s="68" t="n"/>
+      <c r="G1" s="68" t="n"/>
+      <c r="H1" s="68" t="n"/>
+      <c r="I1" s="68" t="n"/>
+      <c r="J1" s="68" t="n"/>
+      <c r="K1" s="68" t="n"/>
+    </row>
     <row r="2" ht="30" customHeight="1">
-      <c r="A2" s="1" t="inlineStr">
+      <c r="A2" s="69" t="inlineStr">
         <is>
           <t>Customer Requirement Report</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="B2" s="68" t="n"/>
+      <c r="C2" s="68" t="n"/>
+      <c r="D2" s="68" t="n"/>
+      <c r="E2" s="68" t="n"/>
+      <c r="F2" s="70" t="inlineStr">
         <is>
           <t>HumanSoft</t>
         </is>
       </c>
+      <c r="G2" s="68" t="n"/>
+      <c r="H2" s="68" t="n"/>
+      <c r="I2" s="68" t="n"/>
+      <c r="J2" s="68" t="n"/>
+      <c r="K2" s="68" t="n"/>
     </row>
     <row r="3">
-      <c r="F3" s="4" t="inlineStr">
+      <c r="A3" s="68" t="n"/>
+      <c r="B3" s="68" t="n"/>
+      <c r="C3" s="68" t="n"/>
+      <c r="D3" s="68" t="n"/>
+      <c r="E3" s="68" t="n"/>
+      <c r="F3" s="71" t="inlineStr">
         <is>
           <t>FM-SE-03</t>
         </is>
       </c>
+      <c r="G3" s="68" t="n"/>
+      <c r="H3" s="68" t="n"/>
+      <c r="I3" s="68" t="n"/>
+      <c r="J3" s="68" t="n"/>
+      <c r="K3" s="68" t="n"/>
     </row>
     <row r="4">
-      <c r="F4" s="5" t="inlineStr">
+      <c r="A4" s="68" t="n"/>
+      <c r="B4" s="68" t="n"/>
+      <c r="C4" s="68" t="n"/>
+      <c r="D4" s="68" t="n"/>
+      <c r="E4" s="68" t="n"/>
+      <c r="F4" s="72" t="inlineStr">
         <is>
           <t>วันที่เริ่มใช้/ แก้ไข : 02 กุมภาพันธ์ 2569/ 00</t>
         </is>
       </c>
+      <c r="G4" s="68" t="n"/>
+      <c r="H4" s="68" t="n"/>
+      <c r="I4" s="68" t="n"/>
+      <c r="J4" s="68" t="n"/>
+      <c r="K4" s="68" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="68" t="n"/>
+      <c r="B5" s="68" t="n"/>
+      <c r="C5" s="68" t="n"/>
+      <c r="D5" s="68" t="n"/>
+      <c r="E5" s="68" t="n"/>
+      <c r="F5" s="68" t="n"/>
+      <c r="G5" s="68" t="n"/>
+      <c r="H5" s="68" t="n"/>
+      <c r="I5" s="68" t="n"/>
+      <c r="J5" s="68" t="n"/>
+      <c r="K5" s="68" t="n"/>
     </row>
     <row r="6" ht="18" customHeight="1">
-      <c r="A6" s="6" t="inlineStr">
+      <c r="A6" s="73" t="inlineStr">
         <is>
           <t>Domain</t>
         </is>
       </c>
-      <c r="C6" s="8" t="inlineStr">
+      <c r="B6" s="68" t="n"/>
+      <c r="C6" s="74" t="inlineStr">
         <is>
           <t>ทดสอบ</t>
         </is>
       </c>
+      <c r="D6" s="68" t="n"/>
+      <c r="E6" s="68" t="n"/>
+      <c r="F6" s="68" t="n"/>
+      <c r="G6" s="68" t="n"/>
+      <c r="H6" s="68" t="n"/>
+      <c r="I6" s="68" t="n"/>
+      <c r="J6" s="68" t="n"/>
+      <c r="K6" s="68" t="n"/>
     </row>
     <row r="7" ht="18" customHeight="1">
-      <c r="A7" s="6" t="inlineStr">
+      <c r="A7" s="73" t="inlineStr">
         <is>
           <t>บริษัท (Company)</t>
         </is>
       </c>
-      <c r="C7" s="8" t="inlineStr">
+      <c r="B7" s="68" t="n"/>
+      <c r="C7" s="74" t="inlineStr">
         <is>
           <t>ทดสอบ</t>
         </is>
       </c>
+      <c r="D7" s="68" t="n"/>
+      <c r="E7" s="68" t="n"/>
+      <c r="F7" s="68" t="n"/>
+      <c r="G7" s="68" t="n"/>
+      <c r="H7" s="68" t="n"/>
+      <c r="I7" s="68" t="n"/>
+      <c r="J7" s="68" t="n"/>
+      <c r="K7" s="68" t="n"/>
     </row>
     <row r="8" ht="18" customHeight="1">
-      <c r="A8" s="6" t="inlineStr">
+      <c r="A8" s="73" t="inlineStr">
         <is>
           <t>วันที่อัปเดต</t>
         </is>
       </c>
-      <c r="C8" s="8" t="inlineStr">
+      <c r="B8" s="68" t="n"/>
+      <c r="C8" s="74" t="inlineStr">
         <is>
           <t>23/5/2026</t>
         </is>
       </c>
+      <c r="D8" s="68" t="n"/>
+      <c r="E8" s="68" t="n"/>
+      <c r="F8" s="68" t="n"/>
+      <c r="G8" s="68" t="n"/>
+      <c r="H8" s="68" t="n"/>
+      <c r="I8" s="68" t="n"/>
+      <c r="J8" s="68" t="n"/>
+      <c r="K8" s="68" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="68" t="n"/>
+      <c r="B9" s="68" t="n"/>
+      <c r="C9" s="68" t="n"/>
+      <c r="D9" s="68" t="n"/>
+      <c r="E9" s="68" t="n"/>
+      <c r="F9" s="68" t="n"/>
+      <c r="G9" s="68" t="n"/>
+      <c r="H9" s="68" t="n"/>
+      <c r="I9" s="68" t="n"/>
+      <c r="J9" s="68" t="n"/>
+      <c r="K9" s="68" t="n"/>
     </row>
     <row r="10" ht="22" customHeight="1">
-      <c r="A10" s="9" t="inlineStr">
+      <c r="A10" s="75" t="inlineStr">
         <is>
           <t xml:space="preserve">    🎯  สรุป Pain Point หลัก</t>
         </is>
       </c>
+      <c r="B10" s="68" t="n"/>
+      <c r="C10" s="68" t="n"/>
+      <c r="D10" s="68" t="n"/>
+      <c r="E10" s="68" t="n"/>
+      <c r="F10" s="68" t="n"/>
+      <c r="G10" s="68" t="n"/>
+      <c r="H10" s="68" t="n"/>
+      <c r="I10" s="68" t="n"/>
+      <c r="J10" s="68" t="n"/>
+      <c r="K10" s="68" t="n"/>
     </row>
     <row r="11" ht="28" customHeight="1">
-      <c r="A11" s="11" t="inlineStr">
+      <c r="A11" s="76" t="inlineStr">
         <is>
           <t>No.</t>
         </is>
       </c>
-      <c r="B11" s="11" t="inlineStr">
+      <c r="B11" s="76" t="inlineStr">
         <is>
           <t>Requirement / ความต้องการ</t>
         </is>
       </c>
-      <c r="C11" s="61" t="n"/>
-      <c r="D11" s="11" t="inlineStr">
+      <c r="C11" s="77" t="n"/>
+      <c r="D11" s="76" t="inlineStr">
         <is>
           <t>รองรับ
 ✓</t>
         </is>
       </c>
-      <c r="E11" s="11" t="inlineStr">
+      <c r="E11" s="76" t="inlineStr">
         <is>
           <t>ยังไม่
 รองรับ</t>
         </is>
       </c>
-      <c r="F11" s="11" t="inlineStr">
+      <c r="F11" s="76" t="inlineStr">
         <is>
           <t>Solutions / แนวทาง</t>
         </is>
       </c>
-      <c r="G11" s="62" t="n"/>
-      <c r="H11" s="62" t="n"/>
-      <c r="I11" s="62" t="n"/>
-      <c r="J11" s="62" t="n"/>
-      <c r="K11" s="61" t="n"/>
+      <c r="G11" s="78" t="n"/>
+      <c r="H11" s="78" t="n"/>
+      <c r="I11" s="78" t="n"/>
+      <c r="J11" s="78" t="n"/>
+      <c r="K11" s="77" t="n"/>
     </row>
     <row r="12" ht="22" customHeight="1">
-      <c r="A12" s="13" t="n">
+      <c r="A12" s="79" t="n">
         <v>1</v>
       </c>
-      <c r="B12" s="14" t="inlineStr">
+      <c r="B12" s="80" t="inlineStr">
         <is>
           <t>(ระบุความต้องการของลูกค้า)</t>
         </is>
       </c>
-      <c r="C12" s="61" t="n"/>
-      <c r="D12" s="15" t="n"/>
-      <c r="E12" s="15" t="n"/>
-      <c r="F12" s="15" t="n"/>
-      <c r="G12" s="62" t="n"/>
-      <c r="H12" s="62" t="n"/>
-      <c r="I12" s="62" t="n"/>
-      <c r="J12" s="62" t="n"/>
-      <c r="K12" s="61" t="n"/>
+      <c r="C12" s="77" t="n"/>
+      <c r="D12" s="81" t="n"/>
+      <c r="E12" s="81" t="n"/>
+      <c r="F12" s="81" t="n"/>
+      <c r="G12" s="78" t="n"/>
+      <c r="H12" s="78" t="n"/>
+      <c r="I12" s="78" t="n"/>
+      <c r="J12" s="78" t="n"/>
+      <c r="K12" s="77" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="68" t="n"/>
+      <c r="B13" s="68" t="n"/>
+      <c r="C13" s="68" t="n"/>
+      <c r="D13" s="68" t="n"/>
+      <c r="E13" s="68" t="n"/>
+      <c r="F13" s="68" t="n"/>
+      <c r="G13" s="68" t="n"/>
+      <c r="H13" s="68" t="n"/>
+      <c r="I13" s="68" t="n"/>
+      <c r="J13" s="68" t="n"/>
+      <c r="K13" s="68" t="n"/>
     </row>
     <row r="14" ht="22" customHeight="1">
-      <c r="A14" s="9" t="inlineStr">
+      <c r="A14" s="75" t="inlineStr">
         <is>
           <t xml:space="preserve">    🎁  Special Offers</t>
         </is>
       </c>
+      <c r="B14" s="68" t="n"/>
+      <c r="C14" s="68" t="n"/>
+      <c r="D14" s="68" t="n"/>
+      <c r="E14" s="68" t="n"/>
+      <c r="F14" s="68" t="n"/>
+      <c r="G14" s="68" t="n"/>
+      <c r="H14" s="68" t="n"/>
+      <c r="I14" s="68" t="n"/>
+      <c r="J14" s="68" t="n"/>
+      <c r="K14" s="68" t="n"/>
     </row>
     <row r="15" ht="20" customHeight="1">
-      <c r="A15" s="11" t="inlineStr">
+      <c r="A15" s="76" t="inlineStr">
         <is>
           <t>No.</t>
         </is>
       </c>
-      <c r="B15" s="11" t="inlineStr">
+      <c r="B15" s="76" t="inlineStr">
         <is>
           <t>รายการ</t>
         </is>
       </c>
-      <c r="C15" s="61" t="n"/>
-      <c r="D15" s="11" t="inlineStr">
+      <c r="C15" s="77" t="n"/>
+      <c r="D15" s="76" t="inlineStr">
         <is>
           <t>รายละเอียด</t>
         </is>
       </c>
-      <c r="E15" s="62" t="n"/>
-      <c r="F15" s="62" t="n"/>
-      <c r="G15" s="62" t="n"/>
-      <c r="H15" s="62" t="n"/>
-      <c r="I15" s="62" t="n"/>
-      <c r="J15" s="62" t="n"/>
-      <c r="K15" s="61" t="n"/>
+      <c r="E15" s="78" t="n"/>
+      <c r="F15" s="78" t="n"/>
+      <c r="G15" s="78" t="n"/>
+      <c r="H15" s="78" t="n"/>
+      <c r="I15" s="78" t="n"/>
+      <c r="J15" s="78" t="n"/>
+      <c r="K15" s="77" t="n"/>
     </row>
     <row r="16" ht="24" customHeight="1">
-      <c r="A16" s="13" t="n">
+      <c r="A16" s="79" t="n">
         <v>1</v>
       </c>
-      <c r="B16" s="16" t="inlineStr">
+      <c r="B16" s="82" t="inlineStr">
         <is>
           <t>ข้อเสนอพิเศษ</t>
         </is>
       </c>
-      <c r="C16" s="61" t="n"/>
-      <c r="D16" s="17" t="inlineStr">
+      <c r="C16" s="77" t="n"/>
+      <c r="D16" s="83" t="inlineStr">
         <is>
           <t>สำหรับการสมัครใช้งานแพ็กเกจ (สัญญา 1 ปี) — 10 ฟรี 2 เมื่อชำระภายในเดือน</t>
         </is>
       </c>
-      <c r="E16" s="62" t="n"/>
-      <c r="F16" s="62" t="n"/>
-      <c r="G16" s="62" t="n"/>
-      <c r="H16" s="62" t="n"/>
-      <c r="I16" s="62" t="n"/>
-      <c r="J16" s="62" t="n"/>
-      <c r="K16" s="61" t="n"/>
+      <c r="E16" s="78" t="n"/>
+      <c r="F16" s="78" t="n"/>
+      <c r="G16" s="78" t="n"/>
+      <c r="H16" s="78" t="n"/>
+      <c r="I16" s="78" t="n"/>
+      <c r="J16" s="78" t="n"/>
+      <c r="K16" s="77" t="n"/>
     </row>
     <row r="17" ht="96" customHeight="1">
-      <c r="A17" s="18" t="n">
+      <c r="A17" s="84" t="n">
         <v>2</v>
       </c>
-      <c r="B17" s="19" t="inlineStr">
+      <c r="B17" s="85" t="inlineStr">
         <is>
           <t>บริการ</t>
         </is>
       </c>
-      <c r="C17" s="61" t="n"/>
-      <c r="D17" s="21" t="inlineStr">
+      <c r="C17" s="77" t="n"/>
+      <c r="D17" s="86" t="inlineStr">
         <is>
           <t>• ไม่มีค่า MA
 • ขึ้นระบบให้ฟรี
@@ -1145,339 +1728,372 @@
 • Training ฟรี 3 ครั้ง</t>
         </is>
       </c>
-      <c r="E17" s="62" t="n"/>
-      <c r="F17" s="62" t="n"/>
-      <c r="G17" s="62" t="n"/>
-      <c r="H17" s="62" t="n"/>
-      <c r="I17" s="62" t="n"/>
-      <c r="J17" s="62" t="n"/>
-      <c r="K17" s="61" t="n"/>
+      <c r="E17" s="78" t="n"/>
+      <c r="F17" s="78" t="n"/>
+      <c r="G17" s="78" t="n"/>
+      <c r="H17" s="78" t="n"/>
+      <c r="I17" s="78" t="n"/>
+      <c r="J17" s="78" t="n"/>
+      <c r="K17" s="77" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="68" t="n"/>
+      <c r="B18" s="68" t="n"/>
+      <c r="C18" s="68" t="n"/>
+      <c r="D18" s="68" t="n"/>
+      <c r="E18" s="68" t="n"/>
+      <c r="F18" s="68" t="n"/>
+      <c r="G18" s="68" t="n"/>
+      <c r="H18" s="68" t="n"/>
+      <c r="I18" s="68" t="n"/>
+      <c r="J18" s="68" t="n"/>
+      <c r="K18" s="68" t="n"/>
     </row>
     <row r="19" ht="22" customHeight="1">
-      <c r="A19" s="9" t="inlineStr">
+      <c r="A19" s="75" t="inlineStr">
         <is>
           <t xml:space="preserve">    📅  Timeline</t>
         </is>
       </c>
+      <c r="B19" s="68" t="n"/>
+      <c r="C19" s="68" t="n"/>
+      <c r="D19" s="68" t="n"/>
+      <c r="E19" s="68" t="n"/>
+      <c r="F19" s="68" t="n"/>
+      <c r="G19" s="68" t="n"/>
+      <c r="H19" s="68" t="n"/>
+      <c r="I19" s="68" t="n"/>
+      <c r="J19" s="68" t="n"/>
+      <c r="K19" s="68" t="n"/>
     </row>
     <row r="20" ht="16" customHeight="1">
-      <c r="A20" s="22" t="inlineStr">
+      <c r="A20" s="87" t="inlineStr">
         <is>
           <t>■ HumanSoft        ■ Client        ★ Go live / Paid</t>
         </is>
       </c>
+      <c r="B20" s="68" t="n"/>
+      <c r="C20" s="68" t="n"/>
+      <c r="D20" s="68" t="n"/>
+      <c r="E20" s="68" t="n"/>
+      <c r="F20" s="68" t="n"/>
+      <c r="G20" s="68" t="n"/>
+      <c r="H20" s="68" t="n"/>
+      <c r="I20" s="68" t="n"/>
+      <c r="J20" s="68" t="n"/>
+      <c r="K20" s="68" t="n"/>
     </row>
     <row r="21" ht="18" customHeight="1">
-      <c r="A21" s="23" t="inlineStr">
+      <c r="A21" s="88" t="inlineStr">
         <is>
           <t>Step</t>
         </is>
       </c>
-      <c r="B21" s="63" t="n"/>
-      <c r="C21" s="11" t="inlineStr">
+      <c r="B21" s="89" t="n"/>
+      <c r="C21" s="76" t="inlineStr">
         <is>
           <t>รายการ</t>
         </is>
       </c>
-      <c r="D21" s="25" t="inlineStr">
+      <c r="D21" s="90" t="inlineStr">
         <is>
           <t>Month 1</t>
         </is>
       </c>
-      <c r="E21" s="62" t="n"/>
-      <c r="F21" s="62" t="n"/>
-      <c r="G21" s="61" t="n"/>
-      <c r="H21" s="25" t="inlineStr">
+      <c r="E21" s="78" t="n"/>
+      <c r="F21" s="78" t="n"/>
+      <c r="G21" s="77" t="n"/>
+      <c r="H21" s="90" t="inlineStr">
         <is>
           <t>Month 2</t>
         </is>
       </c>
-      <c r="I21" s="62" t="n"/>
-      <c r="J21" s="62" t="n"/>
-      <c r="K21" s="61" t="n"/>
+      <c r="I21" s="78" t="n"/>
+      <c r="J21" s="78" t="n"/>
+      <c r="K21" s="77" t="n"/>
     </row>
     <row r="22" ht="16" customHeight="1">
-      <c r="A22" s="64" t="n"/>
-      <c r="B22" s="65" t="n"/>
-      <c r="C22" s="66" t="n"/>
-      <c r="D22" s="26" t="inlineStr">
+      <c r="A22" s="91" t="n"/>
+      <c r="B22" s="92" t="n"/>
+      <c r="C22" s="93" t="n"/>
+      <c r="D22" s="94" t="inlineStr">
         <is>
           <t>W1</t>
         </is>
       </c>
-      <c r="E22" s="26" t="inlineStr">
+      <c r="E22" s="94" t="inlineStr">
         <is>
           <t>W2</t>
         </is>
       </c>
-      <c r="F22" s="26" t="inlineStr">
+      <c r="F22" s="94" t="inlineStr">
         <is>
           <t>W3</t>
         </is>
       </c>
-      <c r="G22" s="26" t="inlineStr">
+      <c r="G22" s="94" t="inlineStr">
         <is>
           <t>W4</t>
         </is>
       </c>
-      <c r="H22" s="26" t="inlineStr">
+      <c r="H22" s="94" t="inlineStr">
         <is>
           <t>W1</t>
         </is>
       </c>
-      <c r="I22" s="26" t="inlineStr">
+      <c r="I22" s="94" t="inlineStr">
         <is>
           <t>W2</t>
         </is>
       </c>
-      <c r="J22" s="26" t="inlineStr">
+      <c r="J22" s="94" t="inlineStr">
         <is>
           <t>W3</t>
         </is>
       </c>
-      <c r="K22" s="26" t="inlineStr">
+      <c r="K22" s="94" t="inlineStr">
         <is>
           <t>W4</t>
         </is>
       </c>
     </row>
     <row r="23" ht="22" customHeight="1">
-      <c r="A23" s="27" t="inlineStr">
+      <c r="A23" s="95" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="B23" s="28" t="inlineStr">
+      <c r="B23" s="96" t="inlineStr">
         <is>
           <t>Demo</t>
         </is>
       </c>
-      <c r="C23" s="29" t="inlineStr">
+      <c r="C23" s="97" t="inlineStr">
         <is>
           <t>Demo</t>
         </is>
       </c>
-      <c r="D23" s="30" t="inlineStr">
+      <c r="D23" s="98" t="inlineStr">
         <is>
           <t>▶</t>
         </is>
       </c>
-      <c r="E23" s="30" t="inlineStr">
+      <c r="E23" s="98" t="inlineStr">
         <is>
           <t>◀</t>
         </is>
       </c>
-      <c r="F23" s="15" t="n"/>
-      <c r="G23" s="15" t="n"/>
-      <c r="H23" s="15" t="n"/>
-      <c r="I23" s="15" t="n"/>
-      <c r="J23" s="15" t="n"/>
-      <c r="K23" s="15" t="n"/>
+      <c r="F23" s="81" t="n"/>
+      <c r="G23" s="81" t="n"/>
+      <c r="H23" s="81" t="n"/>
+      <c r="I23" s="81" t="n"/>
+      <c r="J23" s="81" t="n"/>
+      <c r="K23" s="81" t="n"/>
     </row>
     <row r="24" ht="22" customHeight="1">
-      <c r="A24" s="67" t="n"/>
-      <c r="B24" s="67" t="n"/>
-      <c r="C24" s="29" t="inlineStr">
+      <c r="A24" s="99" t="n"/>
+      <c r="B24" s="99" t="n"/>
+      <c r="C24" s="97" t="inlineStr">
         <is>
           <t>พิจารณา / Consider</t>
         </is>
       </c>
-      <c r="D24" s="15" t="n"/>
-      <c r="E24" s="31" t="inlineStr">
+      <c r="D24" s="81" t="n"/>
+      <c r="E24" s="100" t="inlineStr">
         <is>
           <t>▶</t>
         </is>
       </c>
-      <c r="F24" s="32" t="n"/>
-      <c r="G24" s="31" t="inlineStr">
+      <c r="F24" s="101" t="n"/>
+      <c r="G24" s="100" t="inlineStr">
         <is>
           <t>◀</t>
         </is>
       </c>
-      <c r="H24" s="15" t="n"/>
-      <c r="I24" s="15" t="n"/>
-      <c r="J24" s="15" t="n"/>
-      <c r="K24" s="15" t="n"/>
+      <c r="H24" s="81" t="n"/>
+      <c r="I24" s="81" t="n"/>
+      <c r="J24" s="81" t="n"/>
+      <c r="K24" s="81" t="n"/>
     </row>
     <row r="25" ht="22" customHeight="1">
-      <c r="A25" s="66" t="n"/>
-      <c r="B25" s="66" t="n"/>
-      <c r="C25" s="29" t="inlineStr">
+      <c r="A25" s="93" t="n"/>
+      <c r="B25" s="93" t="n"/>
+      <c r="C25" s="97" t="inlineStr">
         <is>
           <t>ชำระเงิน / Paid</t>
         </is>
       </c>
-      <c r="D25" s="33" t="n"/>
-      <c r="E25" s="33" t="n"/>
-      <c r="F25" s="33" t="n"/>
-      <c r="G25" s="31" t="inlineStr">
+      <c r="D25" s="102" t="n"/>
+      <c r="E25" s="102" t="n"/>
+      <c r="F25" s="102" t="n"/>
+      <c r="G25" s="100" t="inlineStr">
         <is>
           <t>★</t>
         </is>
       </c>
-      <c r="H25" s="33" t="n"/>
-      <c r="I25" s="33" t="n"/>
-      <c r="J25" s="33" t="n"/>
-      <c r="K25" s="33" t="n"/>
+      <c r="H25" s="102" t="n"/>
+      <c r="I25" s="102" t="n"/>
+      <c r="J25" s="102" t="n"/>
+      <c r="K25" s="102" t="n"/>
     </row>
     <row r="26" ht="22" customHeight="1">
-      <c r="A26" s="27" t="inlineStr">
+      <c r="A26" s="95" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="B26" s="28" t="inlineStr">
+      <c r="B26" s="96" t="inlineStr">
         <is>
           <t>Implement</t>
         </is>
       </c>
-      <c r="C26" s="29" t="inlineStr">
+      <c r="C26" s="97" t="inlineStr">
         <is>
           <t>การเตรียมข้อมูลสำหรับการขึ้นระบบ</t>
         </is>
       </c>
-      <c r="D26" s="15" t="n"/>
-      <c r="E26" s="15" t="n"/>
-      <c r="F26" s="15" t="n"/>
-      <c r="G26" s="15" t="n"/>
-      <c r="H26" s="30" t="inlineStr">
+      <c r="D26" s="81" t="n"/>
+      <c r="E26" s="81" t="n"/>
+      <c r="F26" s="81" t="n"/>
+      <c r="G26" s="81" t="n"/>
+      <c r="H26" s="98" t="inlineStr">
         <is>
           <t>▶</t>
         </is>
       </c>
-      <c r="I26" s="30" t="inlineStr">
+      <c r="I26" s="98" t="inlineStr">
         <is>
           <t>◀</t>
         </is>
       </c>
-      <c r="J26" s="15" t="n"/>
-      <c r="K26" s="15" t="n"/>
+      <c r="J26" s="81" t="n"/>
+      <c r="K26" s="81" t="n"/>
     </row>
     <row r="27" ht="22" customHeight="1">
-      <c r="A27" s="67" t="n"/>
-      <c r="B27" s="67" t="n"/>
-      <c r="C27" s="29" t="inlineStr">
+      <c r="A27" s="99" t="n"/>
+      <c r="B27" s="99" t="n"/>
+      <c r="C27" s="97" t="inlineStr">
         <is>
           <t>นำเข้าข้อมูลพนักงาน</t>
         </is>
       </c>
-      <c r="D27" s="15" t="n"/>
-      <c r="E27" s="15" t="n"/>
-      <c r="F27" s="15" t="n"/>
-      <c r="G27" s="15" t="n"/>
-      <c r="H27" s="15" t="n"/>
-      <c r="I27" s="30" t="inlineStr">
+      <c r="D27" s="81" t="n"/>
+      <c r="E27" s="81" t="n"/>
+      <c r="F27" s="81" t="n"/>
+      <c r="G27" s="81" t="n"/>
+      <c r="H27" s="81" t="n"/>
+      <c r="I27" s="98" t="inlineStr">
         <is>
           <t>◆</t>
         </is>
       </c>
-      <c r="J27" s="15" t="n"/>
-      <c r="K27" s="15" t="n"/>
+      <c r="J27" s="81" t="n"/>
+      <c r="K27" s="81" t="n"/>
     </row>
     <row r="28" ht="22" customHeight="1">
-      <c r="A28" s="67" t="n"/>
-      <c r="B28" s="67" t="n"/>
-      <c r="C28" s="29" t="inlineStr">
+      <c r="A28" s="99" t="n"/>
+      <c r="B28" s="99" t="n"/>
+      <c r="C28" s="97" t="inlineStr">
         <is>
           <t>การ Setting ระบบ</t>
         </is>
       </c>
-      <c r="D28" s="15" t="n"/>
-      <c r="E28" s="15" t="n"/>
-      <c r="F28" s="15" t="n"/>
-      <c r="G28" s="15" t="n"/>
-      <c r="H28" s="15" t="n"/>
-      <c r="I28" s="30" t="inlineStr">
+      <c r="D28" s="81" t="n"/>
+      <c r="E28" s="81" t="n"/>
+      <c r="F28" s="81" t="n"/>
+      <c r="G28" s="81" t="n"/>
+      <c r="H28" s="81" t="n"/>
+      <c r="I28" s="98" t="inlineStr">
         <is>
           <t>◆</t>
         </is>
       </c>
-      <c r="J28" s="15" t="n"/>
-      <c r="K28" s="15" t="n"/>
+      <c r="J28" s="81" t="n"/>
+      <c r="K28" s="81" t="n"/>
     </row>
     <row r="29" ht="22" customHeight="1">
-      <c r="A29" s="67" t="n"/>
-      <c r="B29" s="67" t="n"/>
-      <c r="C29" s="29" t="inlineStr">
+      <c r="A29" s="99" t="n"/>
+      <c r="B29" s="99" t="n"/>
+      <c r="C29" s="97" t="inlineStr">
         <is>
           <t>Online Training 3 ครั้ง</t>
         </is>
       </c>
-      <c r="D29" s="15" t="n"/>
-      <c r="E29" s="15" t="n"/>
-      <c r="F29" s="15" t="n"/>
-      <c r="G29" s="15" t="n"/>
-      <c r="H29" s="15" t="n"/>
-      <c r="I29" s="30" t="inlineStr">
+      <c r="D29" s="81" t="n"/>
+      <c r="E29" s="81" t="n"/>
+      <c r="F29" s="81" t="n"/>
+      <c r="G29" s="81" t="n"/>
+      <c r="H29" s="81" t="n"/>
+      <c r="I29" s="98" t="inlineStr">
         <is>
           <t>▶</t>
         </is>
       </c>
-      <c r="J29" s="34" t="n"/>
-      <c r="K29" s="30" t="inlineStr">
+      <c r="J29" s="103" t="n"/>
+      <c r="K29" s="98" t="inlineStr">
         <is>
           <t>◀</t>
         </is>
       </c>
     </row>
     <row r="30" ht="22" customHeight="1">
-      <c r="A30" s="67" t="n"/>
-      <c r="B30" s="67" t="n"/>
-      <c r="C30" s="29" t="inlineStr">
+      <c r="A30" s="99" t="n"/>
+      <c r="B30" s="99" t="n"/>
+      <c r="C30" s="97" t="inlineStr">
         <is>
           <t>ทดสอบทำเงินเดือน</t>
         </is>
       </c>
-      <c r="D30" s="15" t="n"/>
-      <c r="E30" s="15" t="n"/>
-      <c r="F30" s="15" t="n"/>
-      <c r="G30" s="15" t="n"/>
-      <c r="H30" s="15" t="n"/>
-      <c r="I30" s="15" t="n"/>
-      <c r="J30" s="30" t="inlineStr">
+      <c r="D30" s="81" t="n"/>
+      <c r="E30" s="81" t="n"/>
+      <c r="F30" s="81" t="n"/>
+      <c r="G30" s="81" t="n"/>
+      <c r="H30" s="81" t="n"/>
+      <c r="I30" s="81" t="n"/>
+      <c r="J30" s="98" t="inlineStr">
         <is>
           <t>◆</t>
         </is>
       </c>
-      <c r="K30" s="15" t="n"/>
+      <c r="K30" s="81" t="n"/>
     </row>
     <row r="31" ht="22" customHeight="1">
-      <c r="A31" s="67" t="n"/>
-      <c r="B31" s="67" t="n"/>
-      <c r="C31" s="29" t="inlineStr">
+      <c r="A31" s="99" t="n"/>
+      <c r="B31" s="99" t="n"/>
+      <c r="C31" s="97" t="inlineStr">
         <is>
           <t>การเตรียมนำเข้าข้อมูลย้อนหลัง</t>
         </is>
       </c>
-      <c r="D31" s="15" t="n"/>
-      <c r="E31" s="15" t="n"/>
-      <c r="F31" s="15" t="n"/>
-      <c r="G31" s="15" t="n"/>
-      <c r="H31" s="15" t="n"/>
-      <c r="I31" s="15" t="n"/>
-      <c r="J31" s="31" t="inlineStr">
+      <c r="D31" s="81" t="n"/>
+      <c r="E31" s="81" t="n"/>
+      <c r="F31" s="81" t="n"/>
+      <c r="G31" s="81" t="n"/>
+      <c r="H31" s="81" t="n"/>
+      <c r="I31" s="81" t="n"/>
+      <c r="J31" s="100" t="inlineStr">
         <is>
           <t>◆</t>
         </is>
       </c>
-      <c r="K31" s="15" t="n"/>
+      <c r="K31" s="81" t="n"/>
     </row>
     <row r="32" ht="22" customHeight="1">
-      <c r="A32" s="66" t="n"/>
-      <c r="B32" s="66" t="n"/>
-      <c r="C32" s="29" t="inlineStr">
+      <c r="A32" s="93" t="n"/>
+      <c r="B32" s="93" t="n"/>
+      <c r="C32" s="97" t="inlineStr">
         <is>
           <t>การนำเข้าข้อมูลย้อนหลัง / Go live</t>
         </is>
       </c>
-      <c r="D32" s="33" t="n"/>
-      <c r="E32" s="33" t="n"/>
-      <c r="F32" s="33" t="n"/>
-      <c r="G32" s="33" t="n"/>
-      <c r="H32" s="33" t="n"/>
-      <c r="I32" s="33" t="n"/>
-      <c r="J32" s="33" t="n"/>
-      <c r="K32" s="31" t="inlineStr">
+      <c r="D32" s="102" t="n"/>
+      <c r="E32" s="102" t="n"/>
+      <c r="F32" s="102" t="n"/>
+      <c r="G32" s="102" t="n"/>
+      <c r="H32" s="102" t="n"/>
+      <c r="I32" s="102" t="n"/>
+      <c r="J32" s="102" t="n"/>
+      <c r="K32" s="100" t="inlineStr">
         <is>
           <t>★</t>
         </is>
@@ -1530,7 +2146,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A2:H11"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3.8" customWidth="1" min="1" max="1"/>
@@ -1543,125 +2159,191 @@
     <col width="7" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
+    <row r="1">
+      <c r="A1" s="68" t="n"/>
+      <c r="B1" s="68" t="n"/>
+      <c r="C1" s="68" t="n"/>
+      <c r="D1" s="68" t="n"/>
+      <c r="E1" s="68" t="n"/>
+      <c r="F1" s="68" t="n"/>
+      <c r="G1" s="68" t="n"/>
+      <c r="H1" s="68" t="n"/>
+    </row>
     <row r="2" ht="24" customHeight="1">
-      <c r="A2" s="35" t="inlineStr">
+      <c r="A2" s="104" t="inlineStr">
         <is>
           <t>💰  ราคา &amp; แพ็กเกจ</t>
         </is>
       </c>
-      <c r="G2" s="36" t="inlineStr">
+      <c r="B2" s="68" t="n"/>
+      <c r="C2" s="68" t="n"/>
+      <c r="D2" s="68" t="n"/>
+      <c r="E2" s="68" t="n"/>
+      <c r="F2" s="68" t="n"/>
+      <c r="G2" s="105" t="inlineStr">
         <is>
           <t>Human</t>
         </is>
       </c>
-      <c r="H2" s="37" t="inlineStr">
+      <c r="H2" s="106" t="inlineStr">
         <is>
           <t>Soft</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="38" t="inlineStr">
+      <c r="A3" s="107" t="inlineStr">
         <is>
           <t xml:space="preserve"> ราย 1 ปี  |  จ่าย 10 ฟรี 2</t>
         </is>
       </c>
+      <c r="B3" s="68" t="n"/>
+      <c r="C3" s="68" t="n"/>
+      <c r="D3" s="68" t="n"/>
+      <c r="E3" s="68" t="n"/>
+      <c r="F3" s="68" t="n"/>
+      <c r="G3" s="68" t="n"/>
+      <c r="H3" s="68" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="68" t="n"/>
+      <c r="B4" s="68" t="n"/>
+      <c r="C4" s="68" t="n"/>
+      <c r="D4" s="68" t="n"/>
+      <c r="E4" s="68" t="n"/>
+      <c r="F4" s="68" t="n"/>
+      <c r="G4" s="68" t="n"/>
+      <c r="H4" s="68" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="39" t="inlineStr">
+      <c r="A5" s="108" t="inlineStr">
         <is>
           <t xml:space="preserve">  📊 สรุปราคา</t>
         </is>
       </c>
+      <c r="B5" s="68" t="n"/>
+      <c r="C5" s="68" t="n"/>
+      <c r="D5" s="68" t="n"/>
+      <c r="E5" s="68" t="n"/>
+      <c r="F5" s="68" t="n"/>
+      <c r="G5" s="68" t="n"/>
+      <c r="H5" s="68" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="12" t="n"/>
-      <c r="B6" s="26" t="inlineStr">
+      <c r="A6" s="109" t="n"/>
+      <c r="B6" s="94" t="inlineStr">
         <is>
           <t>รายการ</t>
         </is>
       </c>
-      <c r="C6" s="26" t="inlineStr">
+      <c r="C6" s="94" t="inlineStr">
         <is>
           <t>ราคา</t>
         </is>
       </c>
-      <c r="D6" s="26" t="inlineStr">
+      <c r="D6" s="94" t="inlineStr">
         <is>
           <t>หมายเหตุ</t>
         </is>
       </c>
+      <c r="E6" s="68" t="n"/>
+      <c r="F6" s="68" t="n"/>
+      <c r="G6" s="68" t="n"/>
+      <c r="H6" s="68" t="n"/>
     </row>
     <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="40" t="n">
+      <c r="A7" s="110" t="n">
         <v>1</v>
       </c>
-      <c r="B7" s="41" t="inlineStr">
+      <c r="B7" s="111" t="inlineStr">
         <is>
           <t>ราคาปกติ (ไม่มีโปร / ราย 1 ปี)</t>
         </is>
       </c>
-      <c r="C7" s="61" t="n"/>
-      <c r="D7" s="13" t="inlineStr">
+      <c r="C7" s="77" t="n"/>
+      <c r="D7" s="79" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
+      <c r="E7" s="68" t="n"/>
+      <c r="F7" s="68" t="n"/>
+      <c r="G7" s="68" t="n"/>
+      <c r="H7" s="68" t="n"/>
     </row>
     <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="42" t="n">
+      <c r="A8" s="112" t="n">
         <v>2</v>
       </c>
-      <c r="B8" s="43" t="inlineStr">
+      <c r="B8" s="113" t="inlineStr">
         <is>
           <t>จ่าย 10 ฟรี 2 เดือน</t>
         </is>
       </c>
-      <c r="C8" s="61" t="n"/>
-      <c r="D8" s="18" t="inlineStr">
+      <c r="C8" s="77" t="n"/>
+      <c r="D8" s="84" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
+      <c r="E8" s="68" t="n"/>
+      <c r="F8" s="68" t="n"/>
+      <c r="G8" s="68" t="n"/>
+      <c r="H8" s="68" t="n"/>
     </row>
     <row r="9" ht="20" customHeight="1">
-      <c r="A9" s="40" t="n">
+      <c r="A9" s="110" t="n">
         <v>3</v>
       </c>
-      <c r="B9" s="41" t="inlineStr">
+      <c r="B9" s="111" t="inlineStr">
         <is>
           <t>💎 ยอดสุทธิ</t>
         </is>
       </c>
-      <c r="C9" s="61" t="n"/>
-      <c r="D9" s="44" t="inlineStr">
+      <c r="C9" s="77" t="n"/>
+      <c r="D9" s="114" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
+      <c r="E9" s="68" t="n"/>
+      <c r="F9" s="68" t="n"/>
+      <c r="G9" s="68" t="n"/>
+      <c r="H9" s="68" t="n"/>
     </row>
     <row r="10" ht="20" customHeight="1">
-      <c r="A10" s="42" t="n">
+      <c r="A10" s="112" t="n">
         <v>4</v>
       </c>
-      <c r="B10" s="43" t="inlineStr">
+      <c r="B10" s="113" t="inlineStr">
         <is>
           <t>ราคาเฉลี่ยต่อเดือน</t>
         </is>
       </c>
-      <c r="C10" s="61" t="n"/>
-      <c r="D10" s="18" t="inlineStr">
+      <c r="C10" s="77" t="n"/>
+      <c r="D10" s="84" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
+      <c r="E10" s="68" t="n"/>
+      <c r="F10" s="68" t="n"/>
+      <c r="G10" s="68" t="n"/>
+      <c r="H10" s="68" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="45" t="inlineStr">
+      <c r="A11" s="115" t="inlineStr">
         <is>
           <t>💚 (กรอกราคาตามแพ็กเกจที่ลูกค้าเลือก)</t>
         </is>
       </c>
+      <c r="B11" s="68" t="n"/>
+      <c r="C11" s="68" t="n"/>
+      <c r="D11" s="68" t="n"/>
+      <c r="E11" s="68" t="n"/>
+      <c r="F11" s="68" t="n"/>
+      <c r="G11" s="68" t="n"/>
+      <c r="H11" s="68" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="8">
@@ -1686,7 +2368,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A2:D56"/>
+  <dimension ref="A1:D56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3.8" customWidth="1" min="1" max="1"/>
@@ -1695,667 +2377,721 @@
     <col width="4.8" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
+    <row r="1">
+      <c r="A1" s="68" t="n"/>
+      <c r="B1" s="68" t="n"/>
+      <c r="C1" s="68" t="n"/>
+      <c r="D1" s="68" t="n"/>
+    </row>
     <row r="2" ht="24" customHeight="1">
-      <c r="A2" s="35" t="inlineStr">
+      <c r="A2" s="104" t="inlineStr">
         <is>
           <t>✅  Features ที่ต้องการใช้งาน</t>
         </is>
       </c>
-      <c r="D2" s="46" t="inlineStr">
+      <c r="B2" s="68" t="n"/>
+      <c r="C2" s="68" t="n"/>
+      <c r="D2" s="116" t="inlineStr">
         <is>
           <t>Soft</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="38" t="inlineStr">
+      <c r="A3" s="107" t="inlineStr">
         <is>
           <t xml:space="preserve">  ✓ = ต้องการใช้งาน</t>
         </is>
       </c>
+      <c r="B3" s="68" t="n"/>
+      <c r="C3" s="68" t="n"/>
+      <c r="D3" s="68" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="68" t="n"/>
+      <c r="B4" s="68" t="n"/>
+      <c r="C4" s="68" t="n"/>
+      <c r="D4" s="68" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="7" t="n"/>
-      <c r="B5" s="47" t="inlineStr">
+      <c r="A5" s="117" t="n"/>
+      <c r="B5" s="118" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="C5" s="48" t="inlineStr">
+      <c r="C5" s="119" t="inlineStr">
         <is>
           <t>ฟีเจอร์ที่เลือก</t>
         </is>
       </c>
+      <c r="D5" s="68" t="n"/>
     </row>
     <row r="6" ht="18" customHeight="1">
-      <c r="A6" s="49" t="inlineStr">
+      <c r="A6" s="120" t="inlineStr">
         <is>
           <t xml:space="preserve">  Channel</t>
         </is>
       </c>
+      <c r="B6" s="68" t="n"/>
+      <c r="C6" s="68" t="n"/>
+      <c r="D6" s="68" t="n"/>
     </row>
     <row r="7" ht="17" customHeight="1">
-      <c r="A7" s="15" t="n"/>
-      <c r="B7" s="50" t="inlineStr">
+      <c r="A7" s="81" t="n"/>
+      <c r="B7" s="121" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="C7" s="41" t="inlineStr">
+      <c r="C7" s="111" t="inlineStr">
         <is>
           <t>Web Browser</t>
         </is>
       </c>
-      <c r="D7" s="61" t="n"/>
+      <c r="D7" s="77" t="n"/>
     </row>
     <row r="8" ht="17" customHeight="1">
-      <c r="A8" s="20" t="n"/>
-      <c r="B8" s="50" t="inlineStr">
+      <c r="A8" s="122" t="n"/>
+      <c r="B8" s="121" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="C8" s="43" t="inlineStr">
+      <c r="C8" s="113" t="inlineStr">
         <is>
           <t>Mobile Application / Line OA</t>
         </is>
       </c>
-      <c r="D8" s="61" t="n"/>
+      <c r="D8" s="77" t="n"/>
     </row>
     <row r="9" ht="18" customHeight="1">
-      <c r="A9" s="49" t="inlineStr">
+      <c r="A9" s="120" t="inlineStr">
         <is>
           <t xml:space="preserve">  โครงสร้างทั่วไป</t>
         </is>
       </c>
+      <c r="B9" s="68" t="n"/>
+      <c r="C9" s="68" t="n"/>
+      <c r="D9" s="68" t="n"/>
     </row>
     <row r="10" ht="17" customHeight="1">
-      <c r="A10" s="15" t="n"/>
-      <c r="B10" s="50" t="inlineStr">
+      <c r="A10" s="81" t="n"/>
+      <c r="B10" s="121" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="C10" s="41" t="inlineStr">
+      <c r="C10" s="111" t="inlineStr">
         <is>
           <t>รองรับหลายนิติบุคคล</t>
         </is>
       </c>
-      <c r="D10" s="61" t="n"/>
+      <c r="D10" s="77" t="n"/>
     </row>
     <row r="11" ht="17" customHeight="1">
-      <c r="A11" s="20" t="n"/>
-      <c r="B11" s="50" t="inlineStr">
+      <c r="A11" s="122" t="n"/>
+      <c r="B11" s="121" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="C11" s="43" t="inlineStr">
+      <c r="C11" s="113" t="inlineStr">
         <is>
           <t>รองรับหลายสาขา</t>
         </is>
       </c>
-      <c r="D11" s="61" t="n"/>
+      <c r="D11" s="77" t="n"/>
     </row>
     <row r="12" ht="17" customHeight="1">
-      <c r="A12" s="15" t="n"/>
-      <c r="B12" s="50" t="inlineStr">
+      <c r="A12" s="81" t="n"/>
+      <c r="B12" s="121" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="C12" s="41" t="inlineStr">
+      <c r="C12" s="111" t="inlineStr">
         <is>
           <t>รองรับ 3 ภาษา (ไทย/อังกฤษ/พม่า)</t>
         </is>
       </c>
-      <c r="D12" s="61" t="n"/>
+      <c r="D12" s="77" t="n"/>
     </row>
     <row r="13" ht="18" customHeight="1">
-      <c r="A13" s="49" t="inlineStr">
+      <c r="A13" s="120" t="inlineStr">
         <is>
           <t xml:space="preserve">  โครงสร้างองค์กร</t>
         </is>
       </c>
+      <c r="B13" s="68" t="n"/>
+      <c r="C13" s="68" t="n"/>
+      <c r="D13" s="68" t="n"/>
     </row>
     <row r="14" ht="17" customHeight="1">
-      <c r="A14" s="15" t="n"/>
-      <c r="B14" s="50" t="inlineStr">
+      <c r="A14" s="81" t="n"/>
+      <c r="B14" s="121" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="C14" s="41" t="inlineStr">
+      <c r="C14" s="111" t="inlineStr">
         <is>
           <t>โครงสร้างองค์กร / โครงสร้างตำแหน่ง</t>
         </is>
       </c>
-      <c r="D14" s="61" t="n"/>
+      <c r="D14" s="77" t="n"/>
     </row>
     <row r="15" ht="17" customHeight="1">
-      <c r="A15" s="20" t="n"/>
-      <c r="B15" s="50" t="inlineStr">
+      <c r="A15" s="122" t="n"/>
+      <c r="B15" s="121" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="C15" s="43" t="inlineStr">
+      <c r="C15" s="113" t="inlineStr">
         <is>
           <t>เก็บประวัติข้อมูลพนักงาน</t>
         </is>
       </c>
-      <c r="D15" s="61" t="n"/>
+      <c r="D15" s="77" t="n"/>
     </row>
     <row r="16" ht="17" customHeight="1">
-      <c r="A16" s="15" t="n"/>
-      <c r="B16" s="50" t="inlineStr">
+      <c r="A16" s="81" t="n"/>
+      <c r="B16" s="121" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="C16" s="41" t="inlineStr">
+      <c r="C16" s="111" t="inlineStr">
         <is>
           <t>รองรับการเก็บไฟล์ไม่จำกัดพื้นที่</t>
         </is>
       </c>
-      <c r="D16" s="61" t="n"/>
+      <c r="D16" s="77" t="n"/>
     </row>
     <row r="17" ht="18" customHeight="1">
-      <c r="A17" s="49" t="inlineStr">
+      <c r="A17" s="120" t="inlineStr">
         <is>
           <t xml:space="preserve">  จัดการสิทธิ์การเข้าถึงข้อมูล</t>
         </is>
       </c>
+      <c r="B17" s="68" t="n"/>
+      <c r="C17" s="68" t="n"/>
+      <c r="D17" s="68" t="n"/>
     </row>
     <row r="18" ht="17" customHeight="1">
-      <c r="A18" s="15" t="n"/>
-      <c r="B18" s="50" t="inlineStr">
+      <c r="A18" s="81" t="n"/>
+      <c r="B18" s="121" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="C18" s="41" t="inlineStr">
+      <c r="C18" s="111" t="inlineStr">
         <is>
           <t>กำหนดสิทธิ์ผู้ดูแลระบบ (ไม่จำกัด User)</t>
         </is>
       </c>
-      <c r="D18" s="61" t="n"/>
+      <c r="D18" s="77" t="n"/>
     </row>
     <row r="19" ht="17" customHeight="1">
-      <c r="A19" s="20" t="n"/>
-      <c r="B19" s="50" t="inlineStr">
+      <c r="A19" s="122" t="n"/>
+      <c r="B19" s="121" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="C19" s="43" t="inlineStr">
+      <c r="C19" s="113" t="inlineStr">
         <is>
           <t>กำหนดสิทธิ์มองเห็น/แก้ไขของแต่ละ User</t>
         </is>
       </c>
-      <c r="D19" s="61" t="n"/>
+      <c r="D19" s="77" t="n"/>
     </row>
     <row r="20" ht="17" customHeight="1">
-      <c r="A20" s="15" t="n"/>
-      <c r="B20" s="50" t="inlineStr">
+      <c r="A20" s="81" t="n"/>
+      <c r="B20" s="121" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="C20" s="41" t="inlineStr">
+      <c r="C20" s="111" t="inlineStr">
         <is>
           <t>จัดกลุ่มผู้ใช้ได้</t>
         </is>
       </c>
-      <c r="D20" s="61" t="n"/>
+      <c r="D20" s="77" t="n"/>
     </row>
     <row r="21" ht="18" customHeight="1">
-      <c r="A21" s="49" t="inlineStr">
+      <c r="A21" s="120" t="inlineStr">
         <is>
           <t xml:space="preserve">  ระบบความปลอดภัย</t>
         </is>
       </c>
+      <c r="B21" s="68" t="n"/>
+      <c r="C21" s="68" t="n"/>
+      <c r="D21" s="68" t="n"/>
     </row>
     <row r="22" ht="17" customHeight="1">
-      <c r="A22" s="15" t="n"/>
-      <c r="B22" s="50" t="inlineStr">
+      <c r="A22" s="81" t="n"/>
+      <c r="B22" s="121" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="C22" s="41" t="inlineStr">
+      <c r="C22" s="111" t="inlineStr">
         <is>
           <t>Strong Password</t>
         </is>
       </c>
-      <c r="D22" s="61" t="n"/>
+      <c r="D22" s="77" t="n"/>
     </row>
     <row r="23" ht="17" customHeight="1">
-      <c r="A23" s="20" t="n"/>
-      <c r="B23" s="50" t="inlineStr">
+      <c r="A23" s="122" t="n"/>
+      <c r="B23" s="121" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="C23" s="43" t="inlineStr">
+      <c r="C23" s="113" t="inlineStr">
         <is>
           <t>PDPA Conceal</t>
         </is>
       </c>
-      <c r="D23" s="61" t="n"/>
+      <c r="D23" s="77" t="n"/>
     </row>
     <row r="24" ht="18" customHeight="1">
-      <c r="A24" s="49" t="inlineStr">
+      <c r="A24" s="120" t="inlineStr">
         <is>
           <t xml:space="preserve">  จัดการกะ</t>
         </is>
       </c>
+      <c r="B24" s="68" t="n"/>
+      <c r="C24" s="68" t="n"/>
+      <c r="D24" s="68" t="n"/>
     </row>
     <row r="25" ht="17" customHeight="1">
-      <c r="A25" s="15" t="n"/>
-      <c r="B25" s="50" t="inlineStr">
+      <c r="A25" s="81" t="n"/>
+      <c r="B25" s="121" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="C25" s="41" t="inlineStr">
+      <c r="C25" s="111" t="inlineStr">
         <is>
           <t>กะได้หลายรูปแบบ (Default / หลายกะ / Excel Import)</t>
         </is>
       </c>
-      <c r="D25" s="61" t="n"/>
+      <c r="D25" s="77" t="n"/>
     </row>
     <row r="26" ht="17" customHeight="1">
-      <c r="A26" s="20" t="n"/>
-      <c r="B26" s="50" t="inlineStr">
+      <c r="A26" s="122" t="n"/>
+      <c r="B26" s="121" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="C26" s="43" t="inlineStr">
+      <c r="C26" s="113" t="inlineStr">
         <is>
           <t>วางแผนกะรายเดือน / รายสัปดาห์</t>
         </is>
       </c>
-      <c r="D26" s="61" t="n"/>
+      <c r="D26" s="77" t="n"/>
     </row>
     <row r="27" ht="17" customHeight="1">
-      <c r="A27" s="15" t="n"/>
-      <c r="B27" s="50" t="inlineStr">
+      <c r="A27" s="81" t="n"/>
+      <c r="B27" s="121" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="C27" s="41" t="inlineStr">
+      <c r="C27" s="111" t="inlineStr">
         <is>
           <t>สิทธิ์จัดกะแบบยืดหยุ่น (HR / หัวหน้า / พนักงาน)</t>
         </is>
       </c>
-      <c r="D27" s="61" t="n"/>
+      <c r="D27" s="77" t="n"/>
     </row>
     <row r="28" ht="18" customHeight="1">
-      <c r="A28" s="49" t="inlineStr">
+      <c r="A28" s="120" t="inlineStr">
         <is>
           <t xml:space="preserve">  ลงเวลาการทำงาน</t>
         </is>
       </c>
+      <c r="B28" s="68" t="n"/>
+      <c r="C28" s="68" t="n"/>
+      <c r="D28" s="68" t="n"/>
     </row>
     <row r="29" ht="17" customHeight="1">
-      <c r="A29" s="15" t="n"/>
-      <c r="B29" s="50" t="inlineStr">
+      <c r="A29" s="81" t="n"/>
+      <c r="B29" s="121" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="C29" s="41" t="inlineStr">
+      <c r="C29" s="111" t="inlineStr">
         <is>
           <t>Face Scan (Face Recognition)</t>
         </is>
       </c>
-      <c r="D29" s="61" t="n"/>
+      <c r="D29" s="77" t="n"/>
     </row>
     <row r="30" ht="17" customHeight="1">
-      <c r="A30" s="20" t="n"/>
-      <c r="B30" s="50" t="inlineStr">
+      <c r="A30" s="122" t="n"/>
+      <c r="B30" s="121" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="C30" s="43" t="inlineStr">
+      <c r="C30" s="113" t="inlineStr">
         <is>
           <t>GPS</t>
         </is>
       </c>
-      <c r="D30" s="61" t="n"/>
+      <c r="D30" s="77" t="n"/>
     </row>
     <row r="31" ht="17" customHeight="1">
-      <c r="A31" s="15" t="n"/>
-      <c r="B31" s="50" t="inlineStr">
+      <c r="A31" s="81" t="n"/>
+      <c r="B31" s="121" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="C31" s="41" t="inlineStr">
+      <c r="C31" s="111" t="inlineStr">
         <is>
           <t>เครื่องสแกนนิ้ว</t>
         </is>
       </c>
-      <c r="D31" s="61" t="n"/>
+      <c r="D31" s="77" t="n"/>
     </row>
     <row r="32" ht="18" customHeight="1">
-      <c r="A32" s="49" t="inlineStr">
+      <c r="A32" s="120" t="inlineStr">
         <is>
           <t xml:space="preserve">  เอกสารและการอนุมัติ</t>
         </is>
       </c>
+      <c r="B32" s="68" t="n"/>
+      <c r="C32" s="68" t="n"/>
+      <c r="D32" s="68" t="n"/>
     </row>
     <row r="33" ht="17" customHeight="1">
-      <c r="A33" s="15" t="n"/>
-      <c r="B33" s="50" t="inlineStr">
+      <c r="A33" s="81" t="n"/>
+      <c r="B33" s="121" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="C33" s="41" t="inlineStr">
+      <c r="C33" s="111" t="inlineStr">
         <is>
           <t>เอกสารพื้นฐาน (ลา / OT / สลับกะ / ขอเพิ่มเวลา)</t>
         </is>
       </c>
-      <c r="D33" s="61" t="n"/>
+      <c r="D33" s="77" t="n"/>
     </row>
     <row r="34" ht="17" customHeight="1">
-      <c r="A34" s="20" t="n"/>
-      <c r="B34" s="50" t="inlineStr">
+      <c r="A34" s="122" t="n"/>
+      <c r="B34" s="121" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="C34" s="43" t="inlineStr">
+      <c r="C34" s="113" t="inlineStr">
         <is>
           <t>เบิกเงินล่วงหน้า</t>
         </is>
       </c>
-      <c r="D34" s="61" t="n"/>
+      <c r="D34" s="77" t="n"/>
     </row>
     <row r="35" ht="17" customHeight="1">
-      <c r="A35" s="15" t="n"/>
-      <c r="B35" s="50" t="inlineStr">
+      <c r="A35" s="81" t="n"/>
+      <c r="B35" s="121" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="C35" s="41" t="inlineStr">
+      <c r="C35" s="111" t="inlineStr">
         <is>
           <t>หนังสือรับรองเงินเดือน</t>
         </is>
       </c>
-      <c r="D35" s="61" t="n"/>
+      <c r="D35" s="77" t="n"/>
     </row>
     <row r="36" ht="17" customHeight="1">
-      <c r="A36" s="20" t="n"/>
-      <c r="B36" s="50" t="inlineStr">
+      <c r="A36" s="122" t="n"/>
+      <c r="B36" s="121" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="C36" s="43" t="inlineStr">
+      <c r="C36" s="113" t="inlineStr">
         <is>
           <t>อนุมัติผ่าน Website</t>
         </is>
       </c>
-      <c r="D36" s="61" t="n"/>
+      <c r="D36" s="77" t="n"/>
     </row>
     <row r="37" ht="17" customHeight="1">
-      <c r="A37" s="15" t="n"/>
-      <c r="B37" s="50" t="inlineStr">
+      <c r="A37" s="81" t="n"/>
+      <c r="B37" s="121" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="C37" s="41" t="inlineStr">
+      <c r="C37" s="111" t="inlineStr">
         <is>
           <t>อนุมัติผ่าน App</t>
         </is>
       </c>
-      <c r="D37" s="61" t="n"/>
+      <c r="D37" s="77" t="n"/>
     </row>
     <row r="38" ht="17" customHeight="1">
-      <c r="A38" s="20" t="n"/>
-      <c r="B38" s="50" t="inlineStr">
+      <c r="A38" s="122" t="n"/>
+      <c r="B38" s="121" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="C38" s="43" t="inlineStr">
+      <c r="C38" s="113" t="inlineStr">
         <is>
           <t>สายการอนุมัติ 3-5 ขั้น</t>
         </is>
       </c>
-      <c r="D38" s="61" t="n"/>
+      <c r="D38" s="77" t="n"/>
     </row>
     <row r="39" ht="18" customHeight="1">
-      <c r="A39" s="49" t="inlineStr">
+      <c r="A39" s="120" t="inlineStr">
         <is>
           <t xml:space="preserve">  การคำนวณเงินเดือน</t>
         </is>
       </c>
+      <c r="B39" s="68" t="n"/>
+      <c r="C39" s="68" t="n"/>
+      <c r="D39" s="68" t="n"/>
     </row>
     <row r="40" ht="17" customHeight="1">
-      <c r="A40" s="15" t="n"/>
-      <c r="B40" s="50" t="inlineStr">
+      <c r="A40" s="81" t="n"/>
+      <c r="B40" s="121" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="C40" s="41" t="inlineStr">
+      <c r="C40" s="111" t="inlineStr">
         <is>
           <t>รายรับ/รายจ่าย (อัตโนมัติ / Manual)</t>
         </is>
       </c>
-      <c r="D40" s="61" t="n"/>
+      <c r="D40" s="77" t="n"/>
     </row>
     <row r="41" ht="17" customHeight="1">
-      <c r="A41" s="20" t="n"/>
-      <c r="B41" s="50" t="inlineStr">
+      <c r="A41" s="122" t="n"/>
+      <c r="B41" s="121" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="C41" s="43" t="inlineStr">
+      <c r="C41" s="113" t="inlineStr">
         <is>
           <t>งวดเงินเดือน สูงสุด 4 งวด</t>
         </is>
       </c>
-      <c r="D41" s="61" t="n"/>
+      <c r="D41" s="77" t="n"/>
     </row>
     <row r="42" ht="17" customHeight="1">
-      <c r="A42" s="15" t="n"/>
-      <c r="B42" s="50" t="inlineStr">
+      <c r="A42" s="81" t="n"/>
+      <c r="B42" s="121" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="C42" s="41" t="inlineStr">
+      <c r="C42" s="111" t="inlineStr">
         <is>
           <t>สลิปเงินเดือน</t>
         </is>
       </c>
-      <c r="D42" s="61" t="n"/>
+      <c r="D42" s="77" t="n"/>
     </row>
     <row r="43" ht="17" customHeight="1">
-      <c r="A43" s="20" t="n"/>
-      <c r="B43" s="50" t="inlineStr">
+      <c r="A43" s="122" t="n"/>
+      <c r="B43" s="121" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="C43" s="43" t="inlineStr">
+      <c r="C43" s="113" t="inlineStr">
         <is>
           <t>Text File นำส่งธนาคาร</t>
         </is>
       </c>
-      <c r="D43" s="61" t="n"/>
+      <c r="D43" s="77" t="n"/>
     </row>
     <row r="44" ht="17" customHeight="1">
-      <c r="A44" s="15" t="n"/>
-      <c r="B44" s="50" t="inlineStr">
+      <c r="A44" s="81" t="n"/>
+      <c r="B44" s="121" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="C44" s="41" t="inlineStr">
+      <c r="C44" s="111" t="inlineStr">
         <is>
           <t>ภาษี / ประกันสังคม / กองทุน</t>
         </is>
       </c>
-      <c r="D44" s="61" t="n"/>
+      <c r="D44" s="77" t="n"/>
     </row>
     <row r="45" ht="17" customHeight="1">
-      <c r="A45" s="20" t="n"/>
-      <c r="B45" s="50" t="inlineStr">
+      <c r="A45" s="122" t="n"/>
+      <c r="B45" s="121" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="C45" s="43" t="inlineStr">
+      <c r="C45" s="113" t="inlineStr">
         <is>
           <t>เบี้ยเลี้ยง / เบี้ยขยัน</t>
         </is>
       </c>
-      <c r="D45" s="61" t="n"/>
+      <c r="D45" s="77" t="n"/>
     </row>
     <row r="46" ht="18" customHeight="1">
-      <c r="A46" s="49" t="inlineStr">
+      <c r="A46" s="120" t="inlineStr">
         <is>
           <t xml:space="preserve">  รายงาน</t>
         </is>
       </c>
+      <c r="B46" s="68" t="n"/>
+      <c r="C46" s="68" t="n"/>
+      <c r="D46" s="68" t="n"/>
     </row>
     <row r="47" ht="17" customHeight="1">
-      <c r="A47" s="15" t="n"/>
-      <c r="B47" s="50" t="inlineStr">
+      <c r="A47" s="81" t="n"/>
+      <c r="B47" s="121" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="C47" s="41" t="inlineStr">
+      <c r="C47" s="111" t="inlineStr">
         <is>
           <t>รายงานมากกว่า 50 แบบ (.pdf / .xlsx / .txt / .dat)</t>
         </is>
       </c>
-      <c r="D47" s="61" t="n"/>
+      <c r="D47" s="77" t="n"/>
     </row>
     <row r="48" ht="18" customHeight="1">
-      <c r="A48" s="49" t="inlineStr">
+      <c r="A48" s="120" t="inlineStr">
         <is>
           <t xml:space="preserve">  การเรียนรู้และพัฒนาองค์กร (HRD)</t>
         </is>
       </c>
+      <c r="B48" s="68" t="n"/>
+      <c r="C48" s="68" t="n"/>
+      <c r="D48" s="68" t="n"/>
     </row>
     <row r="49" ht="17" customHeight="1">
-      <c r="A49" s="15" t="n"/>
-      <c r="B49" s="50" t="inlineStr">
+      <c r="A49" s="81" t="n"/>
+      <c r="B49" s="121" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="C49" s="41" t="inlineStr">
+      <c r="C49" s="111" t="inlineStr">
         <is>
           <t>E-Library / E-Learning</t>
         </is>
       </c>
-      <c r="D49" s="61" t="n"/>
+      <c r="D49" s="77" t="n"/>
     </row>
     <row r="50" ht="17" customHeight="1">
-      <c r="A50" s="20" t="n"/>
-      <c r="B50" s="50" t="inlineStr">
+      <c r="A50" s="122" t="n"/>
+      <c r="B50" s="121" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="C50" s="43" t="inlineStr">
+      <c r="C50" s="113" t="inlineStr">
         <is>
           <t>ประเมินพนักงาน (ไม่จำกัดรอบ)</t>
         </is>
       </c>
-      <c r="D50" s="61" t="n"/>
+      <c r="D50" s="77" t="n"/>
     </row>
     <row r="51" ht="17" customHeight="1">
-      <c r="A51" s="15" t="n"/>
-      <c r="B51" s="50" t="inlineStr">
+      <c r="A51" s="81" t="n"/>
+      <c r="B51" s="121" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="C51" s="41" t="inlineStr">
+      <c r="C51" s="111" t="inlineStr">
         <is>
           <t>KPI Profile</t>
         </is>
       </c>
-      <c r="D51" s="61" t="n"/>
+      <c r="D51" s="77" t="n"/>
     </row>
     <row r="52" ht="17" customHeight="1">
-      <c r="A52" s="20" t="n"/>
-      <c r="B52" s="50" t="inlineStr">
+      <c r="A52" s="122" t="n"/>
+      <c r="B52" s="121" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="C52" s="43" t="inlineStr">
+      <c r="C52" s="113" t="inlineStr">
         <is>
           <t>บันทึกการฝึกอบรม</t>
         </is>
       </c>
-      <c r="D52" s="61" t="n"/>
+      <c r="D52" s="77" t="n"/>
     </row>
     <row r="53" ht="18" customHeight="1">
-      <c r="A53" s="49" t="inlineStr">
+      <c r="A53" s="120" t="inlineStr">
         <is>
           <t xml:space="preserve">  ระบบรับสมัครพนักงาน</t>
         </is>
       </c>
+      <c r="B53" s="68" t="n"/>
+      <c r="C53" s="68" t="n"/>
+      <c r="D53" s="68" t="n"/>
     </row>
     <row r="54" ht="17" customHeight="1">
-      <c r="A54" s="15" t="n"/>
-      <c r="B54" s="50" t="inlineStr">
+      <c r="A54" s="81" t="n"/>
+      <c r="B54" s="121" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="C54" s="41" t="inlineStr">
+      <c r="C54" s="111" t="inlineStr">
         <is>
           <t>ใบสมัครงานออนไลน์</t>
         </is>
       </c>
-      <c r="D54" s="61" t="n"/>
+      <c r="D54" s="77" t="n"/>
     </row>
     <row r="55" ht="17" customHeight="1">
-      <c r="A55" s="20" t="n"/>
-      <c r="B55" s="50" t="inlineStr">
+      <c r="A55" s="122" t="n"/>
+      <c r="B55" s="121" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="C55" s="43" t="inlineStr">
+      <c r="C55" s="113" t="inlineStr">
         <is>
           <t>ระบบติดตามผู้สมัคร</t>
         </is>
       </c>
-      <c r="D55" s="61" t="n"/>
+      <c r="D55" s="77" t="n"/>
     </row>
     <row r="56" ht="17" customHeight="1">
-      <c r="A56" s="15" t="n"/>
-      <c r="B56" s="50" t="inlineStr">
+      <c r="A56" s="81" t="n"/>
+      <c r="B56" s="121" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="C56" s="41" t="inlineStr">
+      <c r="C56" s="111" t="inlineStr">
         <is>
           <t>เอกสารสัญญาจ้าง (ทดลองงาน/บรรจุ)</t>
         </is>
       </c>
-      <c r="D56" s="61" t="n"/>
+      <c r="D56" s="77" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="54">
@@ -2426,6 +3162,225 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
+  <dimension ref="A1:H5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8.800000000000001" customWidth="1" min="1" max="1"/>
+    <col width="16.8" customWidth="1" min="2" max="2"/>
+    <col width="24.8" customWidth="1" min="3" max="3"/>
+    <col width="16.8" customWidth="1" min="4" max="4"/>
+    <col width="12.8" customWidth="1" min="5" max="5"/>
+    <col width="50.8" customWidth="1" min="6" max="6"/>
+    <col width="14.8" customWidth="1" min="7" max="7"/>
+    <col width="30.8" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="123" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="B1" s="123" t="inlineStr">
+        <is>
+          <t>CODE</t>
+        </is>
+      </c>
+      <c r="C1" s="123" t="inlineStr">
+        <is>
+          <t>Topic</t>
+        </is>
+      </c>
+      <c r="D1" s="123" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="E1" s="123" t="inlineStr">
+        <is>
+          <t>Price</t>
+        </is>
+      </c>
+      <c r="F1" s="123" t="inlineStr">
+        <is>
+          <t>Solution</t>
+        </is>
+      </c>
+      <c r="G1" s="123" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="H1" s="123" t="inlineStr">
+        <is>
+          <t>Remark</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="30" customHeight="1">
+      <c r="A2" s="124" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B2" s="125" t="inlineStr">
+        <is>
+          <t>dncaklehiwo;</t>
+        </is>
+      </c>
+      <c r="C2" s="125" t="inlineStr">
+        <is>
+          <t>njfkldfhwqioh;vio</t>
+        </is>
+      </c>
+      <c r="D2" s="126" t="inlineStr">
+        <is>
+          <t>Requirement</t>
+        </is>
+      </c>
+      <c r="E2" s="127" t="inlineStr">
+        <is>
+          <t>฿0.00</t>
+        </is>
+      </c>
+      <c r="F2" s="125" t="inlineStr">
+        <is>
+          <t>fewqnvklhiow;qjiov</t>
+        </is>
+      </c>
+      <c r="G2" s="128" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="H2" s="125" t="n"/>
+    </row>
+    <row r="3" ht="30" customHeight="1">
+      <c r="A3" s="129" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B3" s="130" t="inlineStr">
+        <is>
+          <t>cdwqkvl;hoi;</t>
+        </is>
+      </c>
+      <c r="C3" s="130" t="inlineStr">
+        <is>
+          <t>nfjd,.chnfsjkalhvuk</t>
+        </is>
+      </c>
+      <c r="D3" s="131" t="inlineStr">
+        <is>
+          <t>Fasttrack</t>
+        </is>
+      </c>
+      <c r="E3" s="132" t="inlineStr">
+        <is>
+          <t>฿0.00</t>
+        </is>
+      </c>
+      <c r="F3" s="130" t="inlineStr">
+        <is>
+          <t>ckdlew.qjvkhl;rhejio</t>
+        </is>
+      </c>
+      <c r="G3" s="133" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="H3" s="130" t="n"/>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="124" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B4" s="125" t="inlineStr">
+        <is>
+          <t>c ewqklhvuh</t>
+        </is>
+      </c>
+      <c r="C4" s="125" t="inlineStr">
+        <is>
+          <t>bvnklf.hjiw;h</t>
+        </is>
+      </c>
+      <c r="D4" s="134" t="inlineStr">
+        <is>
+          <t>Customize</t>
+        </is>
+      </c>
+      <c r="E4" s="127" t="inlineStr">
+        <is>
+          <t>฿0.00</t>
+        </is>
+      </c>
+      <c r="F4" s="125" t="inlineStr">
+        <is>
+          <t>fnkdw.dqhvkl;hio</t>
+        </is>
+      </c>
+      <c r="G4" s="135" t="inlineStr">
+        <is>
+          <t>Cancelled</t>
+        </is>
+      </c>
+      <c r="H4" s="125" t="n"/>
+    </row>
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="129" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B5" s="130" t="inlineStr">
+        <is>
+          <t>vndfjeklhioeprh</t>
+        </is>
+      </c>
+      <c r="C5" s="130" t="inlineStr">
+        <is>
+          <t>n,d.ncwklq;iv</t>
+        </is>
+      </c>
+      <c r="D5" s="136" t="inlineStr">
+        <is>
+          <t>Extra Code</t>
+        </is>
+      </c>
+      <c r="E5" s="132" t="inlineStr">
+        <is>
+          <t>฿0.00</t>
+        </is>
+      </c>
+      <c r="F5" s="130" t="inlineStr">
+        <is>
+          <t>nvfl.enqkl;hio;</t>
+        </is>
+      </c>
+      <c r="G5" s="137" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="H5" s="130" t="n"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:K26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -2443,572 +3398,592 @@
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
-      <c r="A1" s="9" t="inlineStr">
+      <c r="A1" s="75" t="inlineStr">
         <is>
           <t xml:space="preserve">    📅  Timeline</t>
         </is>
       </c>
+      <c r="B1" s="68" t="n"/>
+      <c r="C1" s="68" t="n"/>
+      <c r="D1" s="68" t="n"/>
+      <c r="E1" s="68" t="n"/>
+      <c r="F1" s="68" t="n"/>
+      <c r="G1" s="68" t="n"/>
+      <c r="H1" s="68" t="n"/>
+      <c r="I1" s="68" t="n"/>
+      <c r="J1" s="68" t="n"/>
+      <c r="K1" s="68" t="n"/>
     </row>
     <row r="2" ht="16" customHeight="1">
-      <c r="A2" s="22" t="inlineStr">
+      <c r="A2" s="87" t="inlineStr">
         <is>
           <t>■ HumanSoft     ■ Client     ■ HS + Client     ★ Go Live</t>
         </is>
       </c>
+      <c r="B2" s="68" t="n"/>
+      <c r="C2" s="68" t="n"/>
+      <c r="D2" s="68" t="n"/>
+      <c r="E2" s="68" t="n"/>
+      <c r="F2" s="68" t="n"/>
+      <c r="G2" s="68" t="n"/>
+      <c r="H2" s="68" t="n"/>
+      <c r="I2" s="68" t="n"/>
+      <c r="J2" s="68" t="n"/>
+      <c r="K2" s="68" t="n"/>
     </row>
     <row r="3" ht="18" customHeight="1">
-      <c r="A3" s="11" t="inlineStr">
+      <c r="A3" s="76" t="inlineStr">
         <is>
           <t>No.</t>
         </is>
       </c>
-      <c r="B3" s="11" t="inlineStr">
+      <c r="B3" s="76" t="inlineStr">
         <is>
           <t>ผู้รับผิดชอบ</t>
         </is>
       </c>
-      <c r="C3" s="11" t="inlineStr">
+      <c r="C3" s="76" t="inlineStr">
         <is>
           <t>งาน / Task</t>
         </is>
       </c>
-      <c r="D3" s="25" t="inlineStr">
+      <c r="D3" s="90" t="inlineStr">
         <is>
           <t>Month 1</t>
         </is>
       </c>
-      <c r="E3" s="62" t="n"/>
-      <c r="F3" s="62" t="n"/>
-      <c r="G3" s="61" t="n"/>
-      <c r="H3" s="25" t="inlineStr">
+      <c r="E3" s="78" t="n"/>
+      <c r="F3" s="78" t="n"/>
+      <c r="G3" s="77" t="n"/>
+      <c r="H3" s="90" t="inlineStr">
         <is>
           <t>Month 2</t>
         </is>
       </c>
-      <c r="I3" s="62" t="n"/>
-      <c r="J3" s="62" t="n"/>
-      <c r="K3" s="61" t="n"/>
+      <c r="I3" s="78" t="n"/>
+      <c r="J3" s="78" t="n"/>
+      <c r="K3" s="77" t="n"/>
     </row>
     <row r="4" ht="16" customHeight="1">
-      <c r="A4" s="66" t="n"/>
-      <c r="B4" s="66" t="n"/>
-      <c r="C4" s="66" t="n"/>
-      <c r="D4" s="26" t="inlineStr">
+      <c r="A4" s="93" t="n"/>
+      <c r="B4" s="93" t="n"/>
+      <c r="C4" s="93" t="n"/>
+      <c r="D4" s="94" t="inlineStr">
         <is>
           <t>W1</t>
         </is>
       </c>
-      <c r="E4" s="26" t="inlineStr">
+      <c r="E4" s="94" t="inlineStr">
         <is>
           <t>W2</t>
         </is>
       </c>
-      <c r="F4" s="26" t="inlineStr">
+      <c r="F4" s="94" t="inlineStr">
         <is>
           <t>W3</t>
         </is>
       </c>
-      <c r="G4" s="26" t="inlineStr">
+      <c r="G4" s="94" t="inlineStr">
         <is>
           <t>W4</t>
         </is>
       </c>
-      <c r="H4" s="26" t="inlineStr">
+      <c r="H4" s="94" t="inlineStr">
         <is>
           <t>W1</t>
         </is>
       </c>
-      <c r="I4" s="26" t="inlineStr">
+      <c r="I4" s="94" t="inlineStr">
         <is>
           <t>W2</t>
         </is>
       </c>
-      <c r="J4" s="26" t="inlineStr">
+      <c r="J4" s="94" t="inlineStr">
         <is>
           <t>W3</t>
         </is>
       </c>
-      <c r="K4" s="26" t="inlineStr">
+      <c r="K4" s="94" t="inlineStr">
         <is>
           <t>W4</t>
         </is>
       </c>
     </row>
     <row r="5" ht="18" customHeight="1">
-      <c r="A5" s="40" t="n">
+      <c r="A5" s="110" t="n">
         <v>1</v>
       </c>
-      <c r="B5" s="52" t="inlineStr">
+      <c r="B5" s="138" t="inlineStr">
         <is>
           <t>HS + Client</t>
         </is>
       </c>
-      <c r="C5" s="29" t="inlineStr">
+      <c r="C5" s="97" t="inlineStr">
         <is>
           <t>นำเสนอและเจรจาราคา (Presentation &amp; Negotiate Price)</t>
         </is>
       </c>
-      <c r="D5" s="53" t="inlineStr">
+      <c r="D5" s="139" t="inlineStr">
         <is>
           <t>▶</t>
         </is>
       </c>
-      <c r="E5" s="15" t="n"/>
-      <c r="F5" s="15" t="n"/>
-      <c r="G5" s="15" t="n"/>
-      <c r="H5" s="15" t="n"/>
-      <c r="I5" s="15" t="n"/>
-      <c r="J5" s="15" t="n"/>
-      <c r="K5" s="15" t="n"/>
+      <c r="E5" s="81" t="n"/>
+      <c r="F5" s="81" t="n"/>
+      <c r="G5" s="81" t="n"/>
+      <c r="H5" s="81" t="n"/>
+      <c r="I5" s="81" t="n"/>
+      <c r="J5" s="81" t="n"/>
+      <c r="K5" s="81" t="n"/>
     </row>
     <row r="6" ht="18" customHeight="1">
-      <c r="A6" s="42" t="n">
+      <c r="A6" s="112" t="n">
         <v>2</v>
       </c>
-      <c r="B6" s="54" t="inlineStr">
+      <c r="B6" s="140" t="inlineStr">
         <is>
           <t>Client</t>
         </is>
       </c>
-      <c r="C6" s="55" t="inlineStr">
+      <c r="C6" s="141" t="inlineStr">
         <is>
           <t>ชำระเงิน (Payment)</t>
         </is>
       </c>
-      <c r="D6" s="20" t="n"/>
-      <c r="E6" s="32" t="n"/>
-      <c r="F6" s="20" t="n"/>
-      <c r="G6" s="20" t="n"/>
-      <c r="H6" s="20" t="n"/>
-      <c r="I6" s="20" t="n"/>
-      <c r="J6" s="20" t="n"/>
-      <c r="K6" s="20" t="n"/>
+      <c r="D6" s="122" t="n"/>
+      <c r="E6" s="101" t="n"/>
+      <c r="F6" s="122" t="n"/>
+      <c r="G6" s="122" t="n"/>
+      <c r="H6" s="122" t="n"/>
+      <c r="I6" s="122" t="n"/>
+      <c r="J6" s="122" t="n"/>
+      <c r="K6" s="122" t="n"/>
     </row>
     <row r="7" ht="17" customHeight="1">
-      <c r="A7" s="56" t="inlineStr">
+      <c r="A7" s="142" t="inlineStr">
         <is>
           <t>●  การเตรียมข้อมูลสำหรับขึ้นระบบ</t>
         </is>
       </c>
-      <c r="B7" s="62" t="n"/>
-      <c r="C7" s="62" t="n"/>
-      <c r="D7" s="62" t="n"/>
-      <c r="E7" s="62" t="n"/>
-      <c r="F7" s="62" t="n"/>
-      <c r="G7" s="62" t="n"/>
-      <c r="H7" s="62" t="n"/>
-      <c r="I7" s="62" t="n"/>
-      <c r="J7" s="62" t="n"/>
-      <c r="K7" s="61" t="n"/>
+      <c r="B7" s="78" t="n"/>
+      <c r="C7" s="78" t="n"/>
+      <c r="D7" s="78" t="n"/>
+      <c r="E7" s="78" t="n"/>
+      <c r="F7" s="78" t="n"/>
+      <c r="G7" s="78" t="n"/>
+      <c r="H7" s="78" t="n"/>
+      <c r="I7" s="78" t="n"/>
+      <c r="J7" s="78" t="n"/>
+      <c r="K7" s="77" t="n"/>
     </row>
     <row r="8" ht="18" customHeight="1">
-      <c r="A8" s="40" t="n">
+      <c r="A8" s="110" t="n">
         <v>3</v>
       </c>
-      <c r="B8" s="54" t="inlineStr">
+      <c r="B8" s="140" t="inlineStr">
         <is>
           <t>Client</t>
         </is>
       </c>
-      <c r="C8" s="29" t="inlineStr">
+      <c r="C8" s="97" t="inlineStr">
         <is>
           <t>ข้อมูลพนักงาน</t>
         </is>
       </c>
-      <c r="D8" s="15" t="n"/>
-      <c r="E8" s="32" t="n"/>
-      <c r="F8" s="32" t="n"/>
-      <c r="G8" s="15" t="n"/>
-      <c r="H8" s="15" t="n"/>
-      <c r="I8" s="15" t="n"/>
-      <c r="J8" s="15" t="n"/>
-      <c r="K8" s="15" t="n"/>
+      <c r="D8" s="81" t="n"/>
+      <c r="E8" s="101" t="n"/>
+      <c r="F8" s="101" t="n"/>
+      <c r="G8" s="81" t="n"/>
+      <c r="H8" s="81" t="n"/>
+      <c r="I8" s="81" t="n"/>
+      <c r="J8" s="81" t="n"/>
+      <c r="K8" s="81" t="n"/>
     </row>
     <row r="9" ht="18" customHeight="1">
-      <c r="A9" s="42" t="n">
+      <c r="A9" s="112" t="n">
         <v>4</v>
       </c>
-      <c r="B9" s="54" t="inlineStr">
+      <c r="B9" s="140" t="inlineStr">
         <is>
           <t>Client</t>
         </is>
       </c>
-      <c r="C9" s="55" t="inlineStr">
+      <c r="C9" s="141" t="inlineStr">
         <is>
           <t>เงินโอการคำนวณเงินเดือน</t>
         </is>
       </c>
-      <c r="D9" s="20" t="n"/>
-      <c r="E9" s="32" t="n"/>
-      <c r="F9" s="32" t="n"/>
-      <c r="G9" s="20" t="n"/>
-      <c r="H9" s="20" t="n"/>
-      <c r="I9" s="20" t="n"/>
-      <c r="J9" s="20" t="n"/>
-      <c r="K9" s="20" t="n"/>
+      <c r="D9" s="122" t="n"/>
+      <c r="E9" s="101" t="n"/>
+      <c r="F9" s="101" t="n"/>
+      <c r="G9" s="122" t="n"/>
+      <c r="H9" s="122" t="n"/>
+      <c r="I9" s="122" t="n"/>
+      <c r="J9" s="122" t="n"/>
+      <c r="K9" s="122" t="n"/>
     </row>
     <row r="10" ht="18" customHeight="1">
-      <c r="A10" s="40" t="n">
+      <c r="A10" s="110" t="n">
         <v>5</v>
       </c>
-      <c r="B10" s="54" t="inlineStr">
+      <c r="B10" s="140" t="inlineStr">
         <is>
           <t>Client</t>
         </is>
       </c>
-      <c r="C10" s="29" t="inlineStr">
+      <c r="C10" s="97" t="inlineStr">
         <is>
           <t>รายรับรายจ่าย</t>
         </is>
       </c>
-      <c r="D10" s="15" t="n"/>
-      <c r="E10" s="15" t="n"/>
-      <c r="F10" s="32" t="n"/>
-      <c r="G10" s="15" t="n"/>
-      <c r="H10" s="15" t="n"/>
-      <c r="I10" s="15" t="n"/>
-      <c r="J10" s="15" t="n"/>
-      <c r="K10" s="15" t="n"/>
+      <c r="D10" s="81" t="n"/>
+      <c r="E10" s="81" t="n"/>
+      <c r="F10" s="101" t="n"/>
+      <c r="G10" s="81" t="n"/>
+      <c r="H10" s="81" t="n"/>
+      <c r="I10" s="81" t="n"/>
+      <c r="J10" s="81" t="n"/>
+      <c r="K10" s="81" t="n"/>
     </row>
     <row r="11" ht="18" customHeight="1">
-      <c r="A11" s="42" t="n">
+      <c r="A11" s="112" t="n">
         <v>6</v>
       </c>
-      <c r="B11" s="54" t="inlineStr">
+      <c r="B11" s="140" t="inlineStr">
         <is>
           <t>Client</t>
         </is>
       </c>
-      <c r="C11" s="55" t="inlineStr">
+      <c r="C11" s="141" t="inlineStr">
         <is>
           <t>ส่งข้อมูลพนักงาน และข้อมูลตั้งค่า</t>
         </is>
       </c>
-      <c r="D11" s="20" t="n"/>
-      <c r="E11" s="20" t="n"/>
-      <c r="F11" s="32" t="n"/>
-      <c r="G11" s="20" t="n"/>
-      <c r="H11" s="20" t="n"/>
-      <c r="I11" s="20" t="n"/>
-      <c r="J11" s="20" t="n"/>
-      <c r="K11" s="20" t="n"/>
+      <c r="D11" s="122" t="n"/>
+      <c r="E11" s="122" t="n"/>
+      <c r="F11" s="101" t="n"/>
+      <c r="G11" s="122" t="n"/>
+      <c r="H11" s="122" t="n"/>
+      <c r="I11" s="122" t="n"/>
+      <c r="J11" s="122" t="n"/>
+      <c r="K11" s="122" t="n"/>
     </row>
     <row r="12" ht="18" customHeight="1">
-      <c r="A12" s="40" t="n">
+      <c r="A12" s="110" t="n">
         <v>7</v>
       </c>
-      <c r="B12" s="57" t="inlineStr">
+      <c r="B12" s="143" t="inlineStr">
         <is>
           <t>HumanSoft</t>
         </is>
       </c>
-      <c r="C12" s="29" t="inlineStr">
+      <c r="C12" s="97" t="inlineStr">
         <is>
           <t>ดำเนินการนำเข้าข้อมูล (ขึ้นระบบ)</t>
         </is>
       </c>
-      <c r="D12" s="15" t="n"/>
-      <c r="E12" s="15" t="n"/>
-      <c r="F12" s="15" t="n"/>
-      <c r="G12" s="34" t="n"/>
-      <c r="H12" s="15" t="n"/>
-      <c r="I12" s="15" t="n"/>
-      <c r="J12" s="15" t="n"/>
-      <c r="K12" s="15" t="n"/>
+      <c r="D12" s="81" t="n"/>
+      <c r="E12" s="81" t="n"/>
+      <c r="F12" s="81" t="n"/>
+      <c r="G12" s="103" t="n"/>
+      <c r="H12" s="81" t="n"/>
+      <c r="I12" s="81" t="n"/>
+      <c r="J12" s="81" t="n"/>
+      <c r="K12" s="81" t="n"/>
     </row>
     <row r="13" ht="18" customHeight="1">
-      <c r="A13" s="42" t="n">
+      <c r="A13" s="112" t="n">
         <v>8</v>
       </c>
-      <c r="B13" s="54" t="inlineStr">
+      <c r="B13" s="140" t="inlineStr">
         <is>
           <t>Client</t>
         </is>
       </c>
-      <c r="C13" s="55" t="inlineStr">
+      <c r="C13" s="141" t="inlineStr">
         <is>
           <t>ตรวจสอบความถูกต้องของข้อมูล</t>
         </is>
       </c>
-      <c r="D13" s="20" t="n"/>
-      <c r="E13" s="20" t="n"/>
-      <c r="F13" s="20" t="n"/>
-      <c r="G13" s="32" t="n"/>
-      <c r="H13" s="20" t="n"/>
-      <c r="I13" s="20" t="n"/>
-      <c r="J13" s="20" t="n"/>
-      <c r="K13" s="20" t="n"/>
+      <c r="D13" s="122" t="n"/>
+      <c r="E13" s="122" t="n"/>
+      <c r="F13" s="122" t="n"/>
+      <c r="G13" s="101" t="n"/>
+      <c r="H13" s="122" t="n"/>
+      <c r="I13" s="122" t="n"/>
+      <c r="J13" s="122" t="n"/>
+      <c r="K13" s="122" t="n"/>
     </row>
     <row r="14" ht="17" customHeight="1">
-      <c r="A14" s="56" t="inlineStr">
+      <c r="A14" s="142" t="inlineStr">
         <is>
           <t>●  นัดการสอนใช้งาน Application / Website</t>
         </is>
       </c>
-      <c r="B14" s="62" t="n"/>
-      <c r="C14" s="62" t="n"/>
-      <c r="D14" s="62" t="n"/>
-      <c r="E14" s="62" t="n"/>
-      <c r="F14" s="62" t="n"/>
-      <c r="G14" s="62" t="n"/>
-      <c r="H14" s="62" t="n"/>
-      <c r="I14" s="62" t="n"/>
-      <c r="J14" s="62" t="n"/>
-      <c r="K14" s="61" t="n"/>
+      <c r="B14" s="78" t="n"/>
+      <c r="C14" s="78" t="n"/>
+      <c r="D14" s="78" t="n"/>
+      <c r="E14" s="78" t="n"/>
+      <c r="F14" s="78" t="n"/>
+      <c r="G14" s="78" t="n"/>
+      <c r="H14" s="78" t="n"/>
+      <c r="I14" s="78" t="n"/>
+      <c r="J14" s="78" t="n"/>
+      <c r="K14" s="77" t="n"/>
     </row>
     <row r="15" ht="18" customHeight="1">
-      <c r="A15" s="40" t="n">
+      <c r="A15" s="110" t="n">
         <v>9</v>
       </c>
-      <c r="B15" s="57" t="inlineStr">
+      <c r="B15" s="143" t="inlineStr">
         <is>
           <t>HumanSoft</t>
         </is>
       </c>
-      <c r="C15" s="29" t="inlineStr">
+      <c r="C15" s="97" t="inlineStr">
         <is>
           <t>สำหรับ HR และผู้เกี่ยวข้อง</t>
         </is>
       </c>
-      <c r="D15" s="15" t="n"/>
-      <c r="E15" s="15" t="n"/>
-      <c r="F15" s="15" t="n"/>
-      <c r="G15" s="15" t="n"/>
-      <c r="H15" s="34" t="n"/>
-      <c r="I15" s="15" t="n"/>
-      <c r="J15" s="15" t="n"/>
-      <c r="K15" s="15" t="n"/>
+      <c r="D15" s="81" t="n"/>
+      <c r="E15" s="81" t="n"/>
+      <c r="F15" s="81" t="n"/>
+      <c r="G15" s="81" t="n"/>
+      <c r="H15" s="103" t="n"/>
+      <c r="I15" s="81" t="n"/>
+      <c r="J15" s="81" t="n"/>
+      <c r="K15" s="81" t="n"/>
     </row>
     <row r="16" ht="17" customHeight="1">
-      <c r="A16" s="56" t="inlineStr">
+      <c r="A16" s="142" t="inlineStr">
         <is>
           <t>●  Internal Training (ด้วยตัวเอง)</t>
         </is>
       </c>
-      <c r="B16" s="62" t="n"/>
-      <c r="C16" s="62" t="n"/>
-      <c r="D16" s="62" t="n"/>
-      <c r="E16" s="62" t="n"/>
-      <c r="F16" s="62" t="n"/>
-      <c r="G16" s="62" t="n"/>
-      <c r="H16" s="62" t="n"/>
-      <c r="I16" s="62" t="n"/>
-      <c r="J16" s="62" t="n"/>
-      <c r="K16" s="61" t="n"/>
+      <c r="B16" s="78" t="n"/>
+      <c r="C16" s="78" t="n"/>
+      <c r="D16" s="78" t="n"/>
+      <c r="E16" s="78" t="n"/>
+      <c r="F16" s="78" t="n"/>
+      <c r="G16" s="78" t="n"/>
+      <c r="H16" s="78" t="n"/>
+      <c r="I16" s="78" t="n"/>
+      <c r="J16" s="78" t="n"/>
+      <c r="K16" s="77" t="n"/>
     </row>
     <row r="17" ht="18" customHeight="1">
-      <c r="A17" s="40" t="n">
+      <c r="A17" s="110" t="n">
         <v>10</v>
       </c>
-      <c r="B17" s="54" t="inlineStr">
+      <c r="B17" s="140" t="inlineStr">
         <is>
           <t>Client</t>
         </is>
       </c>
-      <c r="C17" s="29" t="inlineStr">
+      <c r="C17" s="97" t="inlineStr">
         <is>
           <t>HumanSoft มีผู้สอนการใช้งาน Application</t>
         </is>
       </c>
-      <c r="D17" s="15" t="n"/>
-      <c r="E17" s="15" t="n"/>
-      <c r="F17" s="15" t="n"/>
-      <c r="G17" s="15" t="n"/>
-      <c r="H17" s="34" t="n"/>
-      <c r="I17" s="15" t="n"/>
-      <c r="J17" s="15" t="n"/>
-      <c r="K17" s="15" t="n"/>
+      <c r="D17" s="81" t="n"/>
+      <c r="E17" s="81" t="n"/>
+      <c r="F17" s="81" t="n"/>
+      <c r="G17" s="81" t="n"/>
+      <c r="H17" s="103" t="n"/>
+      <c r="I17" s="81" t="n"/>
+      <c r="J17" s="81" t="n"/>
+      <c r="K17" s="81" t="n"/>
     </row>
     <row r="18" ht="17" customHeight="1">
-      <c r="A18" s="56" t="inlineStr">
+      <c r="A18" s="142" t="inlineStr">
         <is>
           <t>●  เริ่มการใช้งาน (Parallel Run)</t>
         </is>
       </c>
-      <c r="B18" s="62" t="n"/>
-      <c r="C18" s="62" t="n"/>
-      <c r="D18" s="62" t="n"/>
-      <c r="E18" s="62" t="n"/>
-      <c r="F18" s="62" t="n"/>
-      <c r="G18" s="62" t="n"/>
-      <c r="H18" s="62" t="n"/>
-      <c r="I18" s="62" t="n"/>
-      <c r="J18" s="62" t="n"/>
-      <c r="K18" s="61" t="n"/>
+      <c r="B18" s="78" t="n"/>
+      <c r="C18" s="78" t="n"/>
+      <c r="D18" s="78" t="n"/>
+      <c r="E18" s="78" t="n"/>
+      <c r="F18" s="78" t="n"/>
+      <c r="G18" s="78" t="n"/>
+      <c r="H18" s="78" t="n"/>
+      <c r="I18" s="78" t="n"/>
+      <c r="J18" s="78" t="n"/>
+      <c r="K18" s="77" t="n"/>
     </row>
     <row r="19" ht="18" customHeight="1">
-      <c r="A19" s="40" t="n">
+      <c r="A19" s="110" t="n">
         <v>11</v>
       </c>
-      <c r="B19" s="58" t="inlineStr"/>
-      <c r="C19" s="29" t="inlineStr">
+      <c r="B19" s="144" t="inlineStr"/>
+      <c r="C19" s="97" t="inlineStr">
         <is>
           <t>ลงเวลาการทำงาน (Time Attendance)</t>
         </is>
       </c>
-      <c r="D19" s="15" t="n"/>
-      <c r="E19" s="15" t="n"/>
-      <c r="F19" s="15" t="n"/>
-      <c r="G19" s="15" t="n"/>
-      <c r="H19" s="15" t="n"/>
-      <c r="I19" s="34" t="n"/>
-      <c r="J19" s="15" t="n"/>
-      <c r="K19" s="15" t="n"/>
+      <c r="D19" s="81" t="n"/>
+      <c r="E19" s="81" t="n"/>
+      <c r="F19" s="81" t="n"/>
+      <c r="G19" s="81" t="n"/>
+      <c r="H19" s="81" t="n"/>
+      <c r="I19" s="103" t="n"/>
+      <c r="J19" s="81" t="n"/>
+      <c r="K19" s="81" t="n"/>
     </row>
     <row r="20" ht="18" customHeight="1">
-      <c r="A20" s="42" t="n">
+      <c r="A20" s="112" t="n">
         <v>12</v>
       </c>
-      <c r="B20" s="59" t="inlineStr"/>
-      <c r="C20" s="55" t="inlineStr">
+      <c r="B20" s="145" t="inlineStr"/>
+      <c r="C20" s="141" t="inlineStr">
         <is>
           <t>ยืนยันเอกสาร (Document Approval)</t>
         </is>
       </c>
-      <c r="D20" s="20" t="n"/>
-      <c r="E20" s="20" t="n"/>
-      <c r="F20" s="20" t="n"/>
-      <c r="G20" s="20" t="n"/>
-      <c r="H20" s="20" t="n"/>
-      <c r="I20" s="34" t="n"/>
-      <c r="J20" s="20" t="n"/>
-      <c r="K20" s="20" t="n"/>
+      <c r="D20" s="122" t="n"/>
+      <c r="E20" s="122" t="n"/>
+      <c r="F20" s="122" t="n"/>
+      <c r="G20" s="122" t="n"/>
+      <c r="H20" s="122" t="n"/>
+      <c r="I20" s="103" t="n"/>
+      <c r="J20" s="122" t="n"/>
+      <c r="K20" s="122" t="n"/>
     </row>
     <row r="21" ht="18" customHeight="1">
-      <c r="A21" s="40" t="n">
+      <c r="A21" s="110" t="n">
         <v>13</v>
       </c>
-      <c r="B21" s="54" t="inlineStr">
+      <c r="B21" s="140" t="inlineStr">
         <is>
           <t>Client</t>
         </is>
       </c>
-      <c r="C21" s="29" t="inlineStr">
+      <c r="C21" s="97" t="inlineStr">
         <is>
           <t>ตรวจสอบเวลาการทำงาน</t>
         </is>
       </c>
-      <c r="D21" s="15" t="n"/>
-      <c r="E21" s="15" t="n"/>
-      <c r="F21" s="15" t="n"/>
-      <c r="G21" s="15" t="n"/>
-      <c r="H21" s="15" t="n"/>
-      <c r="I21" s="32" t="n"/>
-      <c r="J21" s="32" t="n"/>
-      <c r="K21" s="15" t="n"/>
+      <c r="D21" s="81" t="n"/>
+      <c r="E21" s="81" t="n"/>
+      <c r="F21" s="81" t="n"/>
+      <c r="G21" s="81" t="n"/>
+      <c r="H21" s="81" t="n"/>
+      <c r="I21" s="101" t="n"/>
+      <c r="J21" s="101" t="n"/>
+      <c r="K21" s="81" t="n"/>
     </row>
     <row r="22" ht="18" customHeight="1">
-      <c r="A22" s="42" t="n">
+      <c r="A22" s="112" t="n">
         <v>14</v>
       </c>
-      <c r="B22" s="54" t="inlineStr">
+      <c r="B22" s="140" t="inlineStr">
         <is>
           <t>Client</t>
         </is>
       </c>
-      <c r="C22" s="55" t="inlineStr">
+      <c r="C22" s="141" t="inlineStr">
         <is>
           <t>เริ่มการใช้งานจริง (Go Live)</t>
         </is>
       </c>
-      <c r="D22" s="20" t="n"/>
-      <c r="E22" s="20" t="n"/>
-      <c r="F22" s="20" t="n"/>
-      <c r="G22" s="20" t="n"/>
-      <c r="H22" s="20" t="n"/>
-      <c r="I22" s="20" t="n"/>
-      <c r="J22" s="60" t="inlineStr">
+      <c r="D22" s="122" t="n"/>
+      <c r="E22" s="122" t="n"/>
+      <c r="F22" s="122" t="n"/>
+      <c r="G22" s="122" t="n"/>
+      <c r="H22" s="122" t="n"/>
+      <c r="I22" s="122" t="n"/>
+      <c r="J22" s="146" t="inlineStr">
         <is>
           <t>★</t>
         </is>
       </c>
-      <c r="K22" s="20" t="n"/>
+      <c r="K22" s="122" t="n"/>
     </row>
     <row r="23" ht="17" customHeight="1">
-      <c r="A23" s="56" t="inlineStr">
+      <c r="A23" s="142" t="inlineStr">
         <is>
           <t>●  เตรียมข้อมูลเงินเดือน (ย้อนหลัง)</t>
         </is>
       </c>
-      <c r="B23" s="62" t="n"/>
-      <c r="C23" s="62" t="n"/>
-      <c r="D23" s="62" t="n"/>
-      <c r="E23" s="62" t="n"/>
-      <c r="F23" s="62" t="n"/>
-      <c r="G23" s="62" t="n"/>
-      <c r="H23" s="62" t="n"/>
-      <c r="I23" s="62" t="n"/>
-      <c r="J23" s="62" t="n"/>
-      <c r="K23" s="61" t="n"/>
+      <c r="B23" s="78" t="n"/>
+      <c r="C23" s="78" t="n"/>
+      <c r="D23" s="78" t="n"/>
+      <c r="E23" s="78" t="n"/>
+      <c r="F23" s="78" t="n"/>
+      <c r="G23" s="78" t="n"/>
+      <c r="H23" s="78" t="n"/>
+      <c r="I23" s="78" t="n"/>
+      <c r="J23" s="78" t="n"/>
+      <c r="K23" s="77" t="n"/>
     </row>
     <row r="24" ht="18" customHeight="1">
-      <c r="A24" s="40" t="n">
+      <c r="A24" s="110" t="n">
         <v>15</v>
       </c>
-      <c r="B24" s="54" t="inlineStr">
+      <c r="B24" s="140" t="inlineStr">
         <is>
           <t>Client</t>
         </is>
       </c>
-      <c r="C24" s="29" t="inlineStr">
+      <c r="C24" s="97" t="inlineStr">
         <is>
           <t>ส่งรายงานสรุปผลคำนวณเงินเดือน (Excel) ย้อนหลัง</t>
         </is>
       </c>
-      <c r="D24" s="15" t="n"/>
-      <c r="E24" s="15" t="n"/>
-      <c r="F24" s="15" t="n"/>
-      <c r="G24" s="15" t="n"/>
-      <c r="H24" s="15" t="n"/>
-      <c r="I24" s="15" t="n"/>
-      <c r="J24" s="32" t="n"/>
-      <c r="K24" s="15" t="n"/>
+      <c r="D24" s="81" t="n"/>
+      <c r="E24" s="81" t="n"/>
+      <c r="F24" s="81" t="n"/>
+      <c r="G24" s="81" t="n"/>
+      <c r="H24" s="81" t="n"/>
+      <c r="I24" s="81" t="n"/>
+      <c r="J24" s="101" t="n"/>
+      <c r="K24" s="81" t="n"/>
     </row>
     <row r="25" ht="18" customHeight="1">
-      <c r="A25" s="42" t="n">
+      <c r="A25" s="112" t="n">
         <v>16</v>
       </c>
-      <c r="B25" s="57" t="inlineStr">
+      <c r="B25" s="143" t="inlineStr">
         <is>
           <t>HumanSoft</t>
         </is>
       </c>
-      <c r="C25" s="55" t="inlineStr">
+      <c r="C25" s="141" t="inlineStr">
         <is>
           <t>ดำเนินการนำเข้าข้อมูลคำนวณเงินเดือน (ย้อนหลัง)</t>
         </is>
       </c>
-      <c r="D25" s="20" t="n"/>
-      <c r="E25" s="20" t="n"/>
-      <c r="F25" s="20" t="n"/>
-      <c r="G25" s="20" t="n"/>
-      <c r="H25" s="20" t="n"/>
-      <c r="I25" s="20" t="n"/>
-      <c r="J25" s="20" t="n"/>
-      <c r="K25" s="34" t="n"/>
+      <c r="D25" s="122" t="n"/>
+      <c r="E25" s="122" t="n"/>
+      <c r="F25" s="122" t="n"/>
+      <c r="G25" s="122" t="n"/>
+      <c r="H25" s="122" t="n"/>
+      <c r="I25" s="122" t="n"/>
+      <c r="J25" s="122" t="n"/>
+      <c r="K25" s="103" t="n"/>
     </row>
     <row r="26" ht="18" customHeight="1">
-      <c r="A26" s="40" t="n">
+      <c r="A26" s="110" t="n">
         <v>17</v>
       </c>
-      <c r="B26" s="54" t="inlineStr">
+      <c r="B26" s="140" t="inlineStr">
         <is>
           <t>Client</t>
         </is>
       </c>
-      <c r="C26" s="29" t="inlineStr">
+      <c r="C26" s="97" t="inlineStr">
         <is>
           <t>ตรวจสอบความถูกต้องของข้อมูล</t>
         </is>
       </c>
-      <c r="D26" s="15" t="n"/>
-      <c r="E26" s="15" t="n"/>
-      <c r="F26" s="15" t="n"/>
-      <c r="G26" s="15" t="n"/>
-      <c r="H26" s="15" t="n"/>
-      <c r="I26" s="15" t="n"/>
-      <c r="J26" s="15" t="n"/>
-      <c r="K26" s="32" t="n"/>
+      <c r="D26" s="81" t="n"/>
+      <c r="E26" s="81" t="n"/>
+      <c r="F26" s="81" t="n"/>
+      <c r="G26" s="81" t="n"/>
+      <c r="H26" s="81" t="n"/>
+      <c r="I26" s="81" t="n"/>
+      <c r="J26" s="81" t="n"/>
+      <c r="K26" s="101" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="12">

</xml_diff>